<commit_message>
vault backup: 2026-05-10 17:30:52
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_disclosures.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_disclosures.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;--&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%;(0.0%);&quot;--&quot;"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00;($#,##0.00);&quot;--&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -89,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -102,6 +103,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -234,6 +236,11 @@
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2025; raw=2,515,269,000</t>
       </text>
     </comment>
+    <comment ref="L7" authorId="0" shapeId="0">
+      <text>
+        <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2026; raw=782,615,000</t>
+      </text>
+    </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
         <t>IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest @ FY2022; raw=-152,664,000</t>
@@ -284,1479 +291,1814 @@
         <t>IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest @ FY2025; raw=125,033,000</t>
       </text>
     </comment>
+    <comment ref="L10" authorId="0" shapeId="0">
+      <text>
+        <t>IncomeLossFromContinuingOperationsBeforeIncomeTaxesExtraordinaryItemsNoncontrollingInterest @ Q1 2026; raw=137,536,000</t>
+      </text>
+    </comment>
     <comment ref="B17" authorId="0" shapeId="0">
       <text>
-        <t>Revenues @ FY2021; raw=273,005,000</t>
+        <t>Revenues @ FY2020; raw=95,480,310</t>
       </text>
     </comment>
     <comment ref="C17" authorId="0" shapeId="0">
       <text>
+        <t>Revenues @ Q1 2021; raw=39,003,000</t>
+      </text>
+    </comment>
+    <comment ref="D17" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q2 2021; raw=53,601,000</t>
+      </text>
+    </comment>
+    <comment ref="E17" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q3 2021; raw=84,490,000</t>
+      </text>
+    </comment>
+    <comment ref="F17" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ FY2021; raw=273,004,795</t>
+      </text>
+    </comment>
+    <comment ref="G17" authorId="0" shapeId="0">
+      <text>
         <t>Revenues @ Q1 2022; raw=123,473,000</t>
       </text>
     </comment>
-    <comment ref="D17" authorId="0" shapeId="0">
+    <comment ref="H17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2022; raw=145,409,000</t>
       </text>
     </comment>
-    <comment ref="E17" authorId="0" shapeId="0">
+    <comment ref="I17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2022; raw=179,541,000</t>
       </text>
     </comment>
-    <comment ref="F17" authorId="0" shapeId="0">
+    <comment ref="J17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2022; raw=617,457,000</t>
       </text>
     </comment>
-    <comment ref="G17" authorId="0" shapeId="0">
+    <comment ref="K17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q1 2023; raw=248,552,000</t>
       </text>
     </comment>
-    <comment ref="H17" authorId="0" shapeId="0">
+    <comment ref="L17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2023; raw=310,815,000</t>
       </text>
     </comment>
-    <comment ref="I17" authorId="0" shapeId="0">
+    <comment ref="M17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2023; raw=371,178,000</t>
       </text>
     </comment>
-    <comment ref="J17" authorId="0" shapeId="0">
+    <comment ref="N17" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2023; raw=1,263,341,000</t>
       </text>
     </comment>
-    <comment ref="K17" authorId="0" shapeId="0">
+    <comment ref="O17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2024; raw=339,512,000</t>
       </text>
     </comment>
-    <comment ref="L17" authorId="0" shapeId="0">
+    <comment ref="P17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2024; raw=382,351,000</t>
       </text>
     </comment>
-    <comment ref="M17" authorId="0" shapeId="0">
+    <comment ref="Q17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2024; raw=247,125,000</t>
       </text>
     </comment>
-    <comment ref="N17" authorId="0" shapeId="0">
+    <comment ref="R17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2024; raw=1,280,894,000</t>
       </text>
     </comment>
-    <comment ref="O17" authorId="0" shapeId="0">
+    <comment ref="S17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2025; raw=306,534,000</t>
       </text>
     </comment>
-    <comment ref="P17" authorId="0" shapeId="0">
+    <comment ref="T17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2025; raw=714,459,000</t>
       </text>
     </comment>
-    <comment ref="Q17" authorId="0" shapeId="0">
+    <comment ref="U17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2025; raw=701,990,000</t>
       </text>
     </comment>
-    <comment ref="R17" authorId="0" shapeId="0">
+    <comment ref="V17" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2025; raw=2,422,490,000</t>
       </text>
     </comment>
+    <comment ref="W17" authorId="0" shapeId="0">
+      <text>
+        <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2026; raw=747,316,000</t>
+      </text>
+    </comment>
     <comment ref="B18" authorId="0" shapeId="0">
       <text>
-        <t>Revenues @ FY2021; raw=38,097,000</t>
+        <t>Revenues @ FY2020; raw=33,727,441</t>
       </text>
     </comment>
     <comment ref="C18" authorId="0" shapeId="0">
       <text>
+        <t>Revenues @ Q1 2021; raw=10,368,000</t>
+      </text>
+    </comment>
+    <comment ref="D18" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q2 2021; raw=10,792,000</t>
+      </text>
+    </comment>
+    <comment ref="E18" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q3 2021; raw=9,536,000</t>
+      </text>
+    </comment>
+    <comment ref="F18" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ FY2021; raw=38,097,016</t>
+      </text>
+    </comment>
+    <comment ref="G18" authorId="0" shapeId="0">
+      <text>
         <t>Revenues @ Q1 2022; raw=8,495,000</t>
       </text>
     </comment>
-    <comment ref="D18" authorId="0" shapeId="0">
+    <comment ref="H18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2022; raw=7,280,000</t>
       </text>
     </comment>
-    <comment ref="E18" authorId="0" shapeId="0">
+    <comment ref="I18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2022; raw=7,546,000</t>
       </text>
     </comment>
-    <comment ref="F18" authorId="0" shapeId="0">
+    <comment ref="J18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2022; raw=31,054,000</t>
       </text>
     </comment>
-    <comment ref="G18" authorId="0" shapeId="0">
+    <comment ref="K18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q1 2023; raw=8,652,000</t>
       </text>
     </comment>
-    <comment ref="H18" authorId="0" shapeId="0">
+    <comment ref="L18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2023; raw=11,909,000</t>
       </text>
     </comment>
-    <comment ref="I18" authorId="0" shapeId="0">
+    <comment ref="M18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2023; raw=11,038,000</t>
       </text>
     </comment>
-    <comment ref="J18" authorId="0" shapeId="0">
+    <comment ref="N18" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2023; raw=43,722,000</t>
       </text>
     </comment>
-    <comment ref="K18" authorId="0" shapeId="0">
+    <comment ref="O18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2024; raw=14,142,000</t>
       </text>
     </comment>
-    <comment ref="L18" authorId="0" shapeId="0">
+    <comment ref="P18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2024; raw=16,684,000</t>
       </text>
     </comment>
-    <comment ref="M18" authorId="0" shapeId="0">
+    <comment ref="Q18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2024; raw=16,243,000</t>
       </text>
     </comment>
-    <comment ref="N18" authorId="0" shapeId="0">
+    <comment ref="R18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2024; raw=61,696,000</t>
       </text>
     </comment>
-    <comment ref="O18" authorId="0" shapeId="0">
+    <comment ref="S18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2025; raw=18,659,000</t>
       </text>
     </comment>
-    <comment ref="P18" authorId="0" shapeId="0">
+    <comment ref="T18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2025; raw=18,301,000</t>
       </text>
     </comment>
-    <comment ref="Q18" authorId="0" shapeId="0">
+    <comment ref="U18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2025; raw=17,691,000</t>
       </text>
     </comment>
-    <comment ref="R18" authorId="0" shapeId="0">
+    <comment ref="V18" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2025; raw=72,544,000</t>
       </text>
     </comment>
+    <comment ref="W18" authorId="0" shapeId="0">
+      <text>
+        <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2026; raw=25,354,000</t>
+      </text>
+    </comment>
     <comment ref="B19" authorId="0" shapeId="0">
       <text>
+        <t>Revenues @ FY2020; raw=23,400,000</t>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q1 2021; raw=6,500,000</t>
+      </text>
+    </comment>
+    <comment ref="D19" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q2 2021; raw=7,900,000</t>
+      </text>
+    </comment>
+    <comment ref="E19" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q3 2021; raw=6,500,000</t>
+      </text>
+    </comment>
+    <comment ref="F19" authorId="0" shapeId="0">
+      <text>
         <t>Revenues @ FY2021; raw=26,900,000</t>
       </text>
     </comment>
-    <comment ref="C19" authorId="0" shapeId="0">
+    <comment ref="G19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q1 2022; raw=5,800,000</t>
       </text>
     </comment>
-    <comment ref="D19" authorId="0" shapeId="0">
+    <comment ref="H19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2022; raw=5,100,000</t>
       </text>
     </comment>
-    <comment ref="E19" authorId="0" shapeId="0">
+    <comment ref="I19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2022; raw=5,300,000</t>
       </text>
     </comment>
-    <comment ref="F19" authorId="0" shapeId="0">
+    <comment ref="J19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2022; raw=21,700,000</t>
       </text>
     </comment>
-    <comment ref="G19" authorId="0" shapeId="0">
+    <comment ref="K19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q1 2023; raw=5,500,000</t>
       </text>
     </comment>
-    <comment ref="H19" authorId="0" shapeId="0">
+    <comment ref="L19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2023; raw=7,900,000</t>
       </text>
     </comment>
-    <comment ref="I19" authorId="0" shapeId="0">
+    <comment ref="M19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2023; raw=7,400,000</t>
       </text>
     </comment>
-    <comment ref="J19" authorId="0" shapeId="0">
+    <comment ref="N19" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2023; raw=29,300,000</t>
       </text>
     </comment>
-    <comment ref="K19" authorId="0" shapeId="0">
+    <comment ref="O19" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2024; raw=10,000,000</t>
       </text>
     </comment>
-    <comment ref="L19" authorId="0" shapeId="0">
+    <comment ref="P19" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2024; raw=11,300,000</t>
       </text>
     </comment>
-    <comment ref="M19" authorId="0" shapeId="0">
+    <comment ref="Q19" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2024; raw=9,500,000</t>
       </text>
     </comment>
-    <comment ref="B20" authorId="0" shapeId="0">
+    <comment ref="F20" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2021; raw=2,538,000</t>
       </text>
     </comment>
-    <comment ref="F20" authorId="0" shapeId="0">
+    <comment ref="J20" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2022; raw=3,647,000</t>
       </text>
     </comment>
-    <comment ref="H20" authorId="0" shapeId="0">
+    <comment ref="L20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2023; raw=1,606,000</t>
       </text>
     </comment>
-    <comment ref="I20" authorId="0" shapeId="0">
+    <comment ref="M20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2023; raw=1,247,000</t>
       </text>
     </comment>
-    <comment ref="J20" authorId="0" shapeId="0">
+    <comment ref="N20" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2023; raw=4,755,000</t>
       </text>
     </comment>
-    <comment ref="K20" authorId="0" shapeId="0">
+    <comment ref="O20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2024; raw=675,000</t>
       </text>
     </comment>
-    <comment ref="L20" authorId="0" shapeId="0">
+    <comment ref="P20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2024; raw=860,000</t>
       </text>
     </comment>
-    <comment ref="M20" authorId="0" shapeId="0">
+    <comment ref="Q20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2024; raw=594,000</t>
       </text>
     </comment>
-    <comment ref="N20" authorId="0" shapeId="0">
+    <comment ref="R20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2024; raw=5,658,000</t>
       </text>
     </comment>
-    <comment ref="O20" authorId="0" shapeId="0">
+    <comment ref="S20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2025; raw=2,244,000</t>
       </text>
     </comment>
-    <comment ref="P20" authorId="0" shapeId="0">
+    <comment ref="T20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2025; raw=4,381,000</t>
       </text>
     </comment>
-    <comment ref="Q20" authorId="0" shapeId="0">
+    <comment ref="U20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2025; raw=3,518,000</t>
       </text>
     </comment>
-    <comment ref="R20" authorId="0" shapeId="0">
+    <comment ref="V20" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2025; raw=12,971,000</t>
       </text>
     </comment>
+    <comment ref="W20" authorId="0" shapeId="0">
+      <text>
+        <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2026; raw=6,995,000</t>
+      </text>
+    </comment>
     <comment ref="B21" authorId="0" shapeId="0">
       <text>
-        <t>Revenues @ FY2021; raw=632,000</t>
+        <t>Revenues @ FY2020; raw=425,323</t>
       </text>
     </comment>
     <comment ref="C21" authorId="0" shapeId="0">
       <text>
+        <t>Revenues @ Q1 2021; raw=128,000</t>
+      </text>
+    </comment>
+    <comment ref="D21" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q2 2021; raw=61,000</t>
+      </text>
+    </comment>
+    <comment ref="E21" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q3 2021; raw=177,000</t>
+      </text>
+    </comment>
+    <comment ref="F21" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ FY2021; raw=631,649</t>
+      </text>
+    </comment>
+    <comment ref="G21" authorId="0" shapeId="0">
+      <text>
         <t>Revenues @ Q1 2022; raw=454,000</t>
       </text>
     </comment>
-    <comment ref="D21" authorId="0" shapeId="0">
+    <comment ref="H21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2022; raw=448,000</t>
       </text>
     </comment>
-    <comment ref="E21" authorId="0" shapeId="0">
+    <comment ref="I21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2022; raw=182,000</t>
       </text>
     </comment>
-    <comment ref="F21" authorId="0" shapeId="0">
+    <comment ref="J21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2022; raw=1,446,000</t>
       </text>
     </comment>
-    <comment ref="G21" authorId="0" shapeId="0">
+    <comment ref="K21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q1 2023; raw=1,477,000</t>
       </text>
     </comment>
-    <comment ref="H21" authorId="0" shapeId="0">
+    <comment ref="L21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2023; raw=1,553,000</t>
       </text>
     </comment>
-    <comment ref="I21" authorId="0" shapeId="0">
+    <comment ref="M21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2023; raw=1,294,000</t>
       </text>
     </comment>
-    <comment ref="J21" authorId="0" shapeId="0">
+    <comment ref="N21" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ FY2023; raw=6,196,000</t>
       </text>
     </comment>
-    <comment ref="K21" authorId="0" shapeId="0">
+    <comment ref="O21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2024; raw=1,379,000</t>
       </text>
     </comment>
-    <comment ref="L21" authorId="0" shapeId="0">
+    <comment ref="P21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2024; raw=2,082,000</t>
       </text>
     </comment>
-    <comment ref="M21" authorId="0" shapeId="0">
+    <comment ref="Q21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2024; raw=1,786,000</t>
       </text>
     </comment>
-    <comment ref="N21" authorId="0" shapeId="0">
+    <comment ref="R21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2024; raw=7,382,000</t>
       </text>
     </comment>
-    <comment ref="O21" authorId="0" shapeId="0">
+    <comment ref="S21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2025; raw=1,839,000</t>
       </text>
     </comment>
-    <comment ref="P21" authorId="0" shapeId="0">
+    <comment ref="T21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q2 2025; raw=2,118,000</t>
       </text>
     </comment>
-    <comment ref="Q21" authorId="0" shapeId="0">
+    <comment ref="U21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q3 2025; raw=1,907,000</t>
       </text>
     </comment>
-    <comment ref="R21" authorId="0" shapeId="0">
+    <comment ref="V21" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ FY2025; raw=7,264,000</t>
       </text>
     </comment>
+    <comment ref="W21" authorId="0" shapeId="0">
+      <text>
+        <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2026; raw=2,950,000</t>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ FY2020; raw=1,092,703</t>
+      </text>
+    </comment>
     <comment ref="C22" authorId="0" shapeId="0">
       <text>
+        <t>Revenues @ Q1 2021; raw=536,000</t>
+      </text>
+    </comment>
+    <comment ref="D22" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q2 2021; raw=619,000</t>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ Q3 2021; raw=706,000</t>
+      </text>
+    </comment>
+    <comment ref="F22" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ FY2021; raw=2,538,099</t>
+      </text>
+    </comment>
+    <comment ref="G22" authorId="0" shapeId="0">
+      <text>
         <t>Revenues @ Q1 2022; raw=966,000</t>
       </text>
     </comment>
-    <comment ref="D22" authorId="0" shapeId="0">
+    <comment ref="H22" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2022; raw=883,000</t>
       </text>
     </comment>
-    <comment ref="E22" authorId="0" shapeId="0">
+    <comment ref="I22" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2022; raw=964,000</t>
       </text>
     </comment>
-    <comment ref="G22" authorId="0" shapeId="0">
+    <comment ref="J22" authorId="0" shapeId="0">
+      <text>
+        <t>Revenues @ FY2022; raw=3,647,000</t>
+      </text>
+    </comment>
+    <comment ref="K22" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q1 2023; raw=1,258,000</t>
       </text>
     </comment>
-    <comment ref="H22" authorId="0" shapeId="0">
+    <comment ref="L22" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q2 2023; raw=1,606,000</t>
       </text>
     </comment>
-    <comment ref="I22" authorId="0" shapeId="0">
+    <comment ref="M22" authorId="0" shapeId="0">
       <text>
         <t>Revenues @ Q3 2023; raw=1,247,000</t>
       </text>
     </comment>
-    <comment ref="K22" authorId="0" shapeId="0">
+    <comment ref="O22" authorId="0" shapeId="0">
       <text>
         <t>RevenueFromContractWithCustomerExcludingAssessedTax @ Q1 2024; raw=675,000</t>
       </text>
     </comment>
-    <comment ref="J25" authorId="0" shapeId="0">
+    <comment ref="N25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2023; raw=24,316,000</t>
       </text>
     </comment>
-    <comment ref="L25" authorId="0" shapeId="0">
+    <comment ref="P25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2024; raw=34,894,000</t>
       </text>
     </comment>
-    <comment ref="M25" authorId="0" shapeId="0">
+    <comment ref="Q25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2024; raw=37,023,000</t>
       </text>
     </comment>
-    <comment ref="N25" authorId="0" shapeId="0">
+    <comment ref="R25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=72,115,000</t>
       </text>
     </comment>
-    <comment ref="O25" authorId="0" shapeId="0">
+    <comment ref="S25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q1 2025; raw=73,023,000</t>
       </text>
     </comment>
-    <comment ref="P25" authorId="0" shapeId="0">
+    <comment ref="T25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2025; raw=190,854,000</t>
       </text>
     </comment>
-    <comment ref="Q25" authorId="0" shapeId="0">
+    <comment ref="U25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2025; raw=197,635,000</t>
       </text>
     </comment>
-    <comment ref="R25" authorId="0" shapeId="0">
+    <comment ref="V25" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2025; raw=197,866,000</t>
       </text>
     </comment>
-    <comment ref="J26" authorId="0" shapeId="0">
+    <comment ref="W25" authorId="0" shapeId="0">
+      <text>
+        <t>NoncurrentAssets @ Q1 2026; raw=202,300,000</t>
+      </text>
+    </comment>
+    <comment ref="N26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2023; raw=2,212,000</t>
       </text>
     </comment>
-    <comment ref="L26" authorId="0" shapeId="0">
+    <comment ref="P26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2024; raw=2,550,000</t>
       </text>
     </comment>
-    <comment ref="M26" authorId="0" shapeId="0">
+    <comment ref="Q26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2024; raw=2,663,000</t>
       </text>
     </comment>
-    <comment ref="N26" authorId="0" shapeId="0">
+    <comment ref="R26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=2,523,000</t>
       </text>
     </comment>
-    <comment ref="O26" authorId="0" shapeId="0">
+    <comment ref="S26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q1 2025; raw=3,744,000</t>
       </text>
     </comment>
-    <comment ref="P26" authorId="0" shapeId="0">
+    <comment ref="T26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2025; raw=4,057,000</t>
       </text>
     </comment>
-    <comment ref="Q26" authorId="0" shapeId="0">
+    <comment ref="U26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2025; raw=4,441,000</t>
       </text>
     </comment>
-    <comment ref="R26" authorId="0" shapeId="0">
+    <comment ref="V26" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2025; raw=4,635,000</t>
       </text>
     </comment>
-    <comment ref="N27" authorId="0" shapeId="0">
+    <comment ref="R27" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=17,101,000</t>
       </text>
     </comment>
-    <comment ref="O27" authorId="0" shapeId="0">
+    <comment ref="S27" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q1 2025; raw=18,708,000</t>
       </text>
     </comment>
-    <comment ref="P27" authorId="0" shapeId="0">
+    <comment ref="T27" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2025; raw=19,759,000</t>
       </text>
     </comment>
-    <comment ref="Q27" authorId="0" shapeId="0">
+    <comment ref="U27" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2025; raw=20,201,000</t>
       </text>
     </comment>
-    <comment ref="R27" authorId="0" shapeId="0">
+    <comment ref="V27" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2025; raw=20,263,000</t>
       </text>
     </comment>
-    <comment ref="J28" authorId="0" shapeId="0">
+    <comment ref="N28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2023; raw=12,153,000</t>
       </text>
     </comment>
-    <comment ref="L28" authorId="0" shapeId="0">
+    <comment ref="P28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2024; raw=11,591,000</t>
       </text>
     </comment>
-    <comment ref="M28" authorId="0" shapeId="0">
+    <comment ref="Q28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2024; raw=11,930,000</t>
       </text>
     </comment>
-    <comment ref="N28" authorId="0" shapeId="0">
+    <comment ref="R28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=10,950,000</t>
       </text>
     </comment>
-    <comment ref="O28" authorId="0" shapeId="0">
+    <comment ref="S28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q1 2025; raw=11,261,000</t>
       </text>
     </comment>
-    <comment ref="P28" authorId="0" shapeId="0">
+    <comment ref="T28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2025; raw=12,030,000</t>
       </text>
     </comment>
-    <comment ref="Q28" authorId="0" shapeId="0">
+    <comment ref="U28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2025; raw=12,133,000</t>
       </text>
     </comment>
-    <comment ref="R28" authorId="0" shapeId="0">
+    <comment ref="V28" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2025; raw=12,004,000</t>
       </text>
     </comment>
-    <comment ref="J29" authorId="0" shapeId="0">
+    <comment ref="N29" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2023; raw=14,394,000</t>
       </text>
     </comment>
-    <comment ref="L29" authorId="0" shapeId="0">
+    <comment ref="P29" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2024; raw=14,171,000</t>
       </text>
     </comment>
-    <comment ref="M29" authorId="0" shapeId="0">
+    <comment ref="Q29" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2024; raw=18,477,000</t>
       </text>
     </comment>
-    <comment ref="N29" authorId="0" shapeId="0">
+    <comment ref="R29" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=17,101,000</t>
       </text>
     </comment>
-    <comment ref="J30" authorId="0" shapeId="0">
+    <comment ref="N30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2023; raw=29,000</t>
       </text>
     </comment>
-    <comment ref="L30" authorId="0" shapeId="0">
+    <comment ref="P30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2024; raw=30,000</t>
       </text>
     </comment>
-    <comment ref="M30" authorId="0" shapeId="0">
+    <comment ref="Q30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2024; raw=30,000</t>
       </text>
     </comment>
-    <comment ref="N30" authorId="0" shapeId="0">
+    <comment ref="R30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=29,000</t>
       </text>
     </comment>
-    <comment ref="O30" authorId="0" shapeId="0">
+    <comment ref="S30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q1 2025; raw=30,000</t>
       </text>
     </comment>
-    <comment ref="P30" authorId="0" shapeId="0">
+    <comment ref="T30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2025; raw=29,000</t>
       </text>
     </comment>
-    <comment ref="Q30" authorId="0" shapeId="0">
+    <comment ref="U30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2025; raw=29,000</t>
       </text>
     </comment>
-    <comment ref="R30" authorId="0" shapeId="0">
+    <comment ref="V30" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2025; raw=29,000</t>
       </text>
     </comment>
-    <comment ref="M31" authorId="0" shapeId="0">
+    <comment ref="V31" authorId="0" shapeId="0">
+      <text>
+        <t>NoncurrentAssets @ FY2025; raw=20,300,000</t>
+      </text>
+    </comment>
+    <comment ref="W31" authorId="0" shapeId="0">
+      <text>
+        <t>NoncurrentAssets @ Q1 2026; raw=21,100,000</t>
+      </text>
+    </comment>
+    <comment ref="Q32" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2024; raw=3,854,000</t>
       </text>
     </comment>
-    <comment ref="N31" authorId="0" shapeId="0">
+    <comment ref="R32" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2024; raw=3,599,000</t>
       </text>
     </comment>
-    <comment ref="O31" authorId="0" shapeId="0">
+    <comment ref="S32" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q1 2025; raw=3,673,000</t>
       </text>
     </comment>
-    <comment ref="P31" authorId="0" shapeId="0">
+    <comment ref="T32" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q2 2025; raw=3,643,000</t>
       </text>
     </comment>
-    <comment ref="Q31" authorId="0" shapeId="0">
+    <comment ref="U32" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ Q3 2025; raw=3,598,000</t>
       </text>
     </comment>
-    <comment ref="R31" authorId="0" shapeId="0">
+    <comment ref="V32" authorId="0" shapeId="0">
       <text>
         <t>NoncurrentAssets @ FY2025; raw=3,595,000</t>
       </text>
     </comment>
-    <comment ref="B38" authorId="0" shapeId="0">
+    <comment ref="B39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="D38" authorId="0" shapeId="0">
+    <comment ref="D39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="E38" authorId="0" shapeId="0">
+    <comment ref="E39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="F38" authorId="0" shapeId="0">
+    <comment ref="F39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2023; raw=1</t>
       </text>
     </comment>
-    <comment ref="G38" authorId="0" shapeId="0">
+    <comment ref="G39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2023; raw=1</t>
       </text>
     </comment>
-    <comment ref="H38" authorId="0" shapeId="0">
+    <comment ref="H39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2023; raw=1</t>
       </text>
     </comment>
-    <comment ref="I38" authorId="0" shapeId="0">
+    <comment ref="I39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2023; raw=1</t>
       </text>
     </comment>
-    <comment ref="J38" authorId="0" shapeId="0">
+    <comment ref="J39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2024; raw=1</t>
       </text>
     </comment>
-    <comment ref="K38" authorId="0" shapeId="0">
+    <comment ref="K39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2024; raw=1</t>
       </text>
     </comment>
-    <comment ref="L38" authorId="0" shapeId="0">
+    <comment ref="L39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="M38" authorId="0" shapeId="0">
+    <comment ref="M39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2024; raw=1</t>
       </text>
     </comment>
-    <comment ref="N38" authorId="0" shapeId="0">
+    <comment ref="N39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2025; raw=1</t>
       </text>
     </comment>
-    <comment ref="O38" authorId="0" shapeId="0">
+    <comment ref="O39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="P38" authorId="0" shapeId="0">
+    <comment ref="P39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="Q38" authorId="0" shapeId="0">
+    <comment ref="Q39" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="B39" authorId="0" shapeId="0">
+    <comment ref="R39" authorId="0" shapeId="0">
+      <text>
+        <t>ConcentrationRiskPercentage1 @ Q1 2026; raw=1</t>
+      </text>
+    </comment>
+    <comment ref="B40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2022; raw=1</t>
       </text>
     </comment>
-    <comment ref="C39" authorId="0" shapeId="0">
+    <comment ref="C40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2022; raw=1</t>
       </text>
     </comment>
-    <comment ref="D39" authorId="0" shapeId="0">
+    <comment ref="D40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2022; raw=1</t>
       </text>
     </comment>
-    <comment ref="E39" authorId="0" shapeId="0">
+    <comment ref="E40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="F39" authorId="0" shapeId="0">
+    <comment ref="F40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="G39" authorId="0" shapeId="0">
+    <comment ref="G40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="H39" authorId="0" shapeId="0">
+    <comment ref="H40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="I39" authorId="0" shapeId="0">
+    <comment ref="I40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="J39" authorId="0" shapeId="0">
+    <comment ref="J40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="K39" authorId="0" shapeId="0">
+    <comment ref="K40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="L39" authorId="0" shapeId="0">
+    <comment ref="L40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="M39" authorId="0" shapeId="0">
+    <comment ref="M40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="N39" authorId="0" shapeId="0">
+    <comment ref="N40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="O39" authorId="0" shapeId="0">
+    <comment ref="O40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2025; raw=1</t>
       </text>
     </comment>
-    <comment ref="P39" authorId="0" shapeId="0">
+    <comment ref="P40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="Q39" authorId="0" shapeId="0">
+    <comment ref="Q40" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="B40" authorId="0" shapeId="0">
+    <comment ref="R40" authorId="0" shapeId="0">
+      <text>
+        <t>ConcentrationRiskPercentage1 @ Q1 2026; raw=0</t>
+      </text>
+    </comment>
+    <comment ref="B41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="C40" authorId="0" shapeId="0">
+    <comment ref="C41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="D40" authorId="0" shapeId="0">
+    <comment ref="D41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="E40" authorId="0" shapeId="0">
+    <comment ref="E41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="F40" authorId="0" shapeId="0">
+    <comment ref="F41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="G40" authorId="0" shapeId="0">
+    <comment ref="G41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="H40" authorId="0" shapeId="0">
+    <comment ref="H41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="I40" authorId="0" shapeId="0">
+    <comment ref="I41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="J40" authorId="0" shapeId="0">
+    <comment ref="J41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="K40" authorId="0" shapeId="0">
+    <comment ref="K41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="L40" authorId="0" shapeId="0">
+    <comment ref="L41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="M40" authorId="0" shapeId="0">
+    <comment ref="M41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="N40" authorId="0" shapeId="0">
+    <comment ref="N41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="O40" authorId="0" shapeId="0">
+    <comment ref="O41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q2 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="P40" authorId="0" shapeId="0">
+    <comment ref="P41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="Q40" authorId="0" shapeId="0">
+    <comment ref="Q41" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="B41" authorId="0" shapeId="0">
+    <comment ref="R41" authorId="0" shapeId="0">
+      <text>
+        <t>ConcentrationRiskPercentage1 @ Q1 2026; raw=0</t>
+      </text>
+    </comment>
+    <comment ref="B42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="E41" authorId="0" shapeId="0">
+    <comment ref="E42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2022; raw=0</t>
       </text>
     </comment>
-    <comment ref="F41" authorId="0" shapeId="0">
+    <comment ref="F42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="H41" authorId="0" shapeId="0">
+    <comment ref="H42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="I41" authorId="0" shapeId="0">
+    <comment ref="I42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2023; raw=0</t>
       </text>
     </comment>
-    <comment ref="J41" authorId="0" shapeId="0">
+    <comment ref="J42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="L41" authorId="0" shapeId="0">
+    <comment ref="L42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="M41" authorId="0" shapeId="0">
+    <comment ref="M42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ FY2024; raw=0</t>
       </text>
     </comment>
-    <comment ref="N41" authorId="0" shapeId="0">
+    <comment ref="N42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q1 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="P41" authorId="0" shapeId="0">
+    <comment ref="P42" authorId="0" shapeId="0">
       <text>
         <t>ConcentrationRiskPercentage1 @ Q3 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="C48" authorId="0" shapeId="0">
+    <comment ref="R42" authorId="0" shapeId="0">
+      <text>
+        <t>ConcentrationRiskPercentage1 @ Q1 2026; raw=0</t>
+      </text>
+    </comment>
+    <comment ref="C49" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaRevenue @ Q3 2024; raw=513,912,000</t>
       </text>
     </comment>
-    <comment ref="D48" authorId="0" shapeId="0">
+    <comment ref="D49" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaRevenue @ FY2024; raw=2,317,965,000</t>
       </text>
     </comment>
-    <comment ref="G48" authorId="0" shapeId="0">
+    <comment ref="E49" authorId="0" shapeId="0">
+      <text>
+        <t>BusinessAcquisitionsProFormaRevenue @ Q1 2025; raw=647,397,000</t>
+      </text>
+    </comment>
+    <comment ref="G49" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaRevenue @ Q3 2025; raw=798,496,000</t>
       </text>
     </comment>
-    <comment ref="H48" authorId="0" shapeId="0">
+    <comment ref="H49" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaRevenue @ FY2025; raw=3,003,677,000</t>
       </text>
     </comment>
-    <comment ref="B49" authorId="0" shapeId="0">
+    <comment ref="I49" authorId="0" shapeId="0">
+      <text>
+        <t>BusinessAcquisitionsProFormaRevenue @ Q1 2026; raw=782,615,000</t>
+      </text>
+    </comment>
+    <comment ref="B50" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaRevenue @ Q2 2024; raw=547,650,000</t>
       </text>
     </comment>
-    <comment ref="F49" authorId="0" shapeId="0">
+    <comment ref="F50" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaRevenue @ Q2 2025; raw=739,259,000</t>
       </text>
     </comment>
-    <comment ref="C52" authorId="0" shapeId="0">
+    <comment ref="C53" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaNetIncomeLoss @ Q3 2024; raw=17,015,000</t>
       </text>
     </comment>
-    <comment ref="D52" authorId="0" shapeId="0">
+    <comment ref="D53" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaNetIncomeLoss @ FY2024; raw=147,638,000</t>
       </text>
     </comment>
-    <comment ref="G52" authorId="0" shapeId="0">
+    <comment ref="E53" authorId="0" shapeId="0">
+      <text>
+        <t>BusinessAcquisitionsProFormaNetIncomeLoss @ Q1 2025; raw=98,690,000</t>
+      </text>
+    </comment>
+    <comment ref="G53" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaNetIncomeLoss @ Q3 2025; raw=-51,019,000</t>
       </text>
     </comment>
-    <comment ref="H52" authorId="0" shapeId="0">
+    <comment ref="H53" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaNetIncomeLoss @ FY2025; raw=218,748,000</t>
       </text>
     </comment>
-    <comment ref="B53" authorId="0" shapeId="0">
+    <comment ref="I53" authorId="0" shapeId="0">
+      <text>
+        <t>BusinessAcquisitionsProFormaNetIncomeLoss @ Q1 2026; raw=110,099,000</t>
+      </text>
+    </comment>
+    <comment ref="B54" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaNetIncomeLoss @ Q2 2024; raw=70,659,000</t>
       </text>
     </comment>
-    <comment ref="F53" authorId="0" shapeId="0">
+    <comment ref="F54" authorId="0" shapeId="0">
       <text>
         <t>BusinessAcquisitionsProFormaNetIncomeLoss @ Q2 2025; raw=116,424,000</t>
       </text>
     </comment>
-    <comment ref="E56" authorId="0" shapeId="0">
+    <comment ref="E57" authorId="0" shapeId="0">
       <text>
         <t>BusinessCombinationConsiderationTransferred1 @ Q1 2025; raw=1,775,000,000</t>
       </text>
     </comment>
-    <comment ref="F56" authorId="0" shapeId="0">
+    <comment ref="F57" authorId="0" shapeId="0">
       <text>
         <t>BusinessCombinationConsiderationTransferred1 @ Q2 2025; raw=2,055,589,000</t>
       </text>
     </comment>
-    <comment ref="G57" authorId="0" shapeId="0">
+    <comment ref="G58" authorId="0" shapeId="0">
       <text>
         <t>BusinessCombinationConsiderationTransferred1 @ Q3 2025; raw=307,603,000</t>
       </text>
     </comment>
-    <comment ref="D64" authorId="0" shapeId="0">
+    <comment ref="D65" authorId="0" shapeId="0">
       <text>
         <t>DebtInstrumentCarryingAmount @ Q4 2025; raw=700,000,000</t>
       </text>
     </comment>
-    <comment ref="B67" authorId="0" shapeId="0">
+    <comment ref="B68" authorId="0" shapeId="0">
       <text>
         <t>DebtInstrumentInterestRateEffectivePercentage @ Q2 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="C67" authorId="0" shapeId="0">
+    <comment ref="C68" authorId="0" shapeId="0">
       <text>
         <t>DebtInstrumentInterestRateEffectivePercentage @ Q3 2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="E67" authorId="0" shapeId="0">
+    <comment ref="E68" authorId="0" shapeId="0">
       <text>
         <t>DebtInstrumentInterestRateEffectivePercentage @ FY2025; raw=0</t>
       </text>
     </comment>
-    <comment ref="D74" authorId="0" shapeId="0">
+    <comment ref="F68" authorId="0" shapeId="0">
+      <text>
+        <t>DebtInstrumentInterestRateEffectivePercentage @ Q1 2026; raw=0</t>
+      </text>
+    </comment>
+    <comment ref="F75" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriodWeightedAverageGrantDateFairValue @ FY2022; raw=25</t>
       </text>
     </comment>
-    <comment ref="D75" authorId="0" shapeId="0">
+    <comment ref="F76" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriodWeightedAverageGrantDateFairValue @ FY2022; raw=22</t>
       </text>
     </comment>
-    <comment ref="F75" authorId="0" shapeId="0">
+    <comment ref="H76" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriodWeightedAverageGrantDateFairValue @ FY2023; raw=33</t>
       </text>
     </comment>
-    <comment ref="B78" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2021; raw=1,700,000</t>
-      </text>
-    </comment>
-    <comment ref="C78" authorId="0" shapeId="0">
+    <comment ref="I79" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2024; raw=275,000</t>
+      </text>
+    </comment>
+    <comment ref="J79" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2024; raw=552,000</t>
+      </text>
+    </comment>
+    <comment ref="K79" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2025; raw=1,074,000</t>
+      </text>
+    </comment>
+    <comment ref="L79" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2025; raw=1,628,000</t>
+      </text>
+    </comment>
+    <comment ref="M79" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2026; raw=805,000</t>
+      </text>
+    </comment>
+    <comment ref="C80" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2021; raw=468,000</t>
+      </text>
+    </comment>
+    <comment ref="D80" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2021; raw=573,428</t>
+      </text>
+    </comment>
+    <comment ref="E80" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2022; raw=189,000</t>
       </text>
     </comment>
-    <comment ref="D78" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2022; raw=700,000</t>
-      </text>
-    </comment>
-    <comment ref="E78" authorId="0" shapeId="0">
+    <comment ref="F80" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2022; raw=248</t>
+      </text>
+    </comment>
+    <comment ref="G80" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2023; raw=124,000</t>
       </text>
     </comment>
-    <comment ref="F78" authorId="0" shapeId="0">
+    <comment ref="H80" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2023; raw=468,000</t>
       </text>
     </comment>
-    <comment ref="G78" authorId="0" shapeId="0">
+    <comment ref="I80" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2024; raw=210,000</t>
       </text>
     </comment>
-    <comment ref="H78" authorId="0" shapeId="0">
+    <comment ref="J80" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2024; raw=377,000</t>
       </text>
     </comment>
-    <comment ref="G79" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2024; raw=275,000</t>
-      </text>
-    </comment>
-    <comment ref="H79" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2024; raw=552,000</t>
-      </text>
-    </comment>
-    <comment ref="I79" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2025; raw=1,074,000</t>
-      </text>
-    </comment>
-    <comment ref="J79" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2025; raw=1,628,000</t>
-      </text>
-    </comment>
-    <comment ref="B80" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2021; raw=45,000</t>
-      </text>
-    </comment>
-    <comment ref="D80" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2022; raw=228,000</t>
-      </text>
-    </comment>
-    <comment ref="G80" authorId="0" shapeId="0">
+    <comment ref="D81" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2021; raw=15</t>
+      </text>
+    </comment>
+    <comment ref="F81" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2022; raw=76</t>
+      </text>
+    </comment>
+    <comment ref="I81" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2024; raw=65,000</t>
       </text>
     </comment>
-    <comment ref="H80" authorId="0" shapeId="0">
+    <comment ref="J81" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2024; raw=175,000</t>
       </text>
     </comment>
-    <comment ref="I80" authorId="0" shapeId="0">
+    <comment ref="K81" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2025; raw=142,000</t>
       </text>
     </comment>
-    <comment ref="J80" authorId="0" shapeId="0">
+    <comment ref="L81" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2025; raw=142,000</t>
       </text>
     </comment>
-    <comment ref="C83" authorId="0" shapeId="0">
+    <comment ref="M81" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ Q1 2026; raw=67,000</t>
+      </text>
+    </comment>
+    <comment ref="B82" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2020; raw=175,737</t>
+      </text>
+    </comment>
+    <comment ref="D83" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsGrantsInPeriod @ FY2021; raw=15,468</t>
+      </text>
+    </comment>
+    <comment ref="I86" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2024; raw=510,000</t>
+      </text>
+    </comment>
+    <comment ref="J86" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2024; raw=803,000</t>
+      </text>
+    </comment>
+    <comment ref="K86" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2025; raw=249,000</t>
+      </text>
+    </comment>
+    <comment ref="L86" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2025; raw=470,000</t>
+      </text>
+    </comment>
+    <comment ref="M86" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2026; raw=478,000</t>
+      </text>
+    </comment>
+    <comment ref="D87" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2021; raw=18,758</t>
+      </text>
+    </comment>
+    <comment ref="E87" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2022; raw=111,000</t>
       </text>
     </comment>
-    <comment ref="E83" authorId="0" shapeId="0">
+    <comment ref="F87" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2022; raw=205</t>
+      </text>
+    </comment>
+    <comment ref="G87" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2023; raw=157,000</t>
       </text>
     </comment>
-    <comment ref="F83" authorId="0" shapeId="0">
+    <comment ref="H87" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2023; raw=670,000</t>
       </text>
     </comment>
-    <comment ref="G83" authorId="0" shapeId="0">
+    <comment ref="I87" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2024; raw=510,000</t>
       </text>
     </comment>
-    <comment ref="H83" authorId="0" shapeId="0">
+    <comment ref="J87" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2024; raw=715,000</t>
       </text>
     </comment>
-    <comment ref="G84" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2024; raw=510,000</t>
-      </text>
-    </comment>
-    <comment ref="H84" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2024; raw=803,000</t>
-      </text>
-    </comment>
-    <comment ref="I84" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ Q1 2025; raw=249,000</t>
-      </text>
-    </comment>
-    <comment ref="J84" authorId="0" shapeId="0">
-      <text>
-        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2025; raw=470,000</t>
-      </text>
-    </comment>
-    <comment ref="F85" authorId="0" shapeId="0">
+    <comment ref="F88" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2022; raw=15</t>
+      </text>
+    </comment>
+    <comment ref="H88" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2023; raw=92,000</t>
       </text>
     </comment>
-    <comment ref="H85" authorId="0" shapeId="0">
+    <comment ref="J88" authorId="0" shapeId="0">
       <text>
         <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2024; raw=78,000</t>
       </text>
     </comment>
-    <comment ref="B92" authorId="0" shapeId="0">
+    <comment ref="B89" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2020; raw=170,145</t>
+      </text>
+    </comment>
+    <comment ref="D89" authorId="0" shapeId="0">
+      <text>
+        <t>ShareBasedCompensationArrangementByShareBasedPaymentAwardEquityInstrumentsOtherThanOptionsVestedInPeriod @ FY2021; raw=18,913</t>
+      </text>
+    </comment>
+    <comment ref="B96" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ FY2020; raw=394,418</t>
+      </text>
+    </comment>
+    <comment ref="C96" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ FY2021; raw=3,051,938</t>
+      </text>
+    </comment>
+    <comment ref="D96" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q1 2022; raw=3,561,000</t>
+      </text>
+    </comment>
+    <comment ref="E96" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q2 2022; raw=4,944,000</t>
+      </text>
+    </comment>
+    <comment ref="F96" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q3 2022; raw=5,505,000</t>
+      </text>
+    </comment>
+    <comment ref="G96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2022; raw=9,885,000</t>
       </text>
     </comment>
-    <comment ref="C92" authorId="0" shapeId="0">
+    <comment ref="H96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2023; raw=11,848,000</t>
       </text>
     </comment>
-    <comment ref="D92" authorId="0" shapeId="0">
+    <comment ref="I96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2023; raw=14,962,000</t>
       </text>
     </comment>
-    <comment ref="E92" authorId="0" shapeId="0">
+    <comment ref="J96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2023; raw=18,703,000</t>
       </text>
     </comment>
-    <comment ref="F92" authorId="0" shapeId="0">
+    <comment ref="K96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2023; raw=21,908,000</t>
       </text>
     </comment>
-    <comment ref="G92" authorId="0" shapeId="0">
+    <comment ref="L96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2024; raw=26,110,000</t>
       </text>
     </comment>
-    <comment ref="H92" authorId="0" shapeId="0">
+    <comment ref="M96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2024; raw=34,844,000</t>
       </text>
     </comment>
-    <comment ref="I92" authorId="0" shapeId="0">
+    <comment ref="N96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2024; raw=36,573,000</t>
       </text>
     </comment>
-    <comment ref="J92" authorId="0" shapeId="0">
+    <comment ref="O96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2024; raw=39,231,000</t>
       </text>
     </comment>
-    <comment ref="K92" authorId="0" shapeId="0">
+    <comment ref="P96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2025; raw=43,441,000</t>
       </text>
     </comment>
-    <comment ref="L92" authorId="0" shapeId="0">
+    <comment ref="Q96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2025; raw=52,892,000</t>
       </text>
     </comment>
-    <comment ref="M92" authorId="0" shapeId="0">
+    <comment ref="R96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2025; raw=57,158,000</t>
       </text>
     </comment>
-    <comment ref="N92" authorId="0" shapeId="0">
+    <comment ref="S96" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2025; raw=60,615,000</t>
       </text>
     </comment>
-    <comment ref="B93" authorId="0" shapeId="0">
+    <comment ref="B97" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ FY2020; raw=78,124</t>
+      </text>
+    </comment>
+    <comment ref="C97" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ FY2021; raw=304,210</t>
+      </text>
+    </comment>
+    <comment ref="D97" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q1 2022; raw=456,000</t>
+      </text>
+    </comment>
+    <comment ref="E97" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q2 2022; raw=739,000</t>
+      </text>
+    </comment>
+    <comment ref="F97" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q3 2022; raw=1,013,000</t>
+      </text>
+    </comment>
+    <comment ref="G97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2022; raw=1,257,000</t>
       </text>
     </comment>
-    <comment ref="C93" authorId="0" shapeId="0">
+    <comment ref="H97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2023; raw=1,524,000</t>
       </text>
     </comment>
-    <comment ref="D93" authorId="0" shapeId="0">
+    <comment ref="I97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2023; raw=2,596,000</t>
       </text>
     </comment>
-    <comment ref="E93" authorId="0" shapeId="0">
+    <comment ref="J97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2023; raw=4,617,000</t>
       </text>
     </comment>
-    <comment ref="F93" authorId="0" shapeId="0">
+    <comment ref="K97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2023; raw=6,143,000</t>
       </text>
     </comment>
-    <comment ref="G93" authorId="0" shapeId="0">
+    <comment ref="L97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2024; raw=6,294,000</t>
       </text>
     </comment>
-    <comment ref="H93" authorId="0" shapeId="0">
+    <comment ref="M97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2024; raw=6,687,000</t>
       </text>
     </comment>
-    <comment ref="I93" authorId="0" shapeId="0">
+    <comment ref="N97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2024; raw=9,070,000</t>
       </text>
     </comment>
-    <comment ref="J93" authorId="0" shapeId="0">
+    <comment ref="O97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2024; raw=12,237,000</t>
       </text>
     </comment>
-    <comment ref="K93" authorId="0" shapeId="0">
+    <comment ref="P97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2025; raw=12,237,000</t>
       </text>
     </comment>
-    <comment ref="L93" authorId="0" shapeId="0">
+    <comment ref="Q97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2025; raw=14,828,000</t>
       </text>
     </comment>
-    <comment ref="M93" authorId="0" shapeId="0">
+    <comment ref="R97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2025; raw=14,919,000</t>
       </text>
     </comment>
-    <comment ref="N93" authorId="0" shapeId="0">
+    <comment ref="S97" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2025; raw=17,501,000</t>
       </text>
     </comment>
-    <comment ref="J94" authorId="0" shapeId="0">
+    <comment ref="O98" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2024; raw=10,136,000</t>
       </text>
     </comment>
-    <comment ref="K94" authorId="0" shapeId="0">
+    <comment ref="P98" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2025; raw=11,683,000</t>
       </text>
     </comment>
-    <comment ref="L94" authorId="0" shapeId="0">
+    <comment ref="Q98" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2025; raw=16,585,000</t>
       </text>
     </comment>
-    <comment ref="M94" authorId="0" shapeId="0">
+    <comment ref="R98" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2025; raw=22,430,000</t>
       </text>
     </comment>
-    <comment ref="N94" authorId="0" shapeId="0">
+    <comment ref="S98" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2025; raw=14,631,000</t>
       </text>
     </comment>
-    <comment ref="B95" authorId="0" shapeId="0">
+    <comment ref="B99" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ FY2020; raw=630,759</t>
+      </text>
+    </comment>
+    <comment ref="C99" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ FY2021; raw=890,695</t>
+      </text>
+    </comment>
+    <comment ref="D99" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q1 2022; raw=968,000</t>
+      </text>
+    </comment>
+    <comment ref="E99" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q2 2022; raw=996,000</t>
+      </text>
+    </comment>
+    <comment ref="F99" authorId="0" shapeId="0">
+      <text>
+        <t>PropertyPlantAndEquipmentGross @ Q3 2022; raw=1,177,000</t>
+      </text>
+    </comment>
+    <comment ref="G99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2022; raw=1,124,000</t>
       </text>
     </comment>
-    <comment ref="C95" authorId="0" shapeId="0">
+    <comment ref="H99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2023; raw=1,158,000</t>
       </text>
     </comment>
-    <comment ref="D95" authorId="0" shapeId="0">
+    <comment ref="I99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2023; raw=1,286,000</t>
       </text>
     </comment>
-    <comment ref="E95" authorId="0" shapeId="0">
+    <comment ref="J99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2023; raw=1,399,000</t>
       </text>
     </comment>
-    <comment ref="F95" authorId="0" shapeId="0">
+    <comment ref="K99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2023; raw=1,467,000</t>
       </text>
     </comment>
-    <comment ref="G95" authorId="0" shapeId="0">
+    <comment ref="L99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2024; raw=1,571,000</t>
       </text>
     </comment>
-    <comment ref="H95" authorId="0" shapeId="0">
+    <comment ref="M99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2024; raw=1,623,000</t>
       </text>
     </comment>
-    <comment ref="I95" authorId="0" shapeId="0">
+    <comment ref="N99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2024; raw=1,632,000</t>
       </text>
     </comment>
-    <comment ref="J95" authorId="0" shapeId="0">
+    <comment ref="O99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2024; raw=2,228,000</t>
       </text>
     </comment>
-    <comment ref="K95" authorId="0" shapeId="0">
+    <comment ref="P99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2025; raw=1,681,000</t>
       </text>
     </comment>
-    <comment ref="L95" authorId="0" shapeId="0">
+    <comment ref="Q99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2025; raw=1,846,000</t>
       </text>
     </comment>
-    <comment ref="M95" authorId="0" shapeId="0">
+    <comment ref="R99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2025; raw=2,880,000</t>
       </text>
     </comment>
-    <comment ref="N95" authorId="0" shapeId="0">
+    <comment ref="S99" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2025; raw=3,570,000</t>
       </text>
     </comment>
-    <comment ref="J96" authorId="0" shapeId="0">
+    <comment ref="O100" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2024; raw=2,561,000</t>
       </text>
     </comment>
-    <comment ref="K96" authorId="0" shapeId="0">
+    <comment ref="P100" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q1 2025; raw=2,375,000</t>
       </text>
     </comment>
-    <comment ref="L96" authorId="0" shapeId="0">
+    <comment ref="Q100" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q2 2025; raw=2,439,000</t>
       </text>
     </comment>
-    <comment ref="M96" authorId="0" shapeId="0">
+    <comment ref="R100" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ Q3 2025; raw=2,443,000</t>
       </text>
     </comment>
-    <comment ref="N96" authorId="0" shapeId="0">
+    <comment ref="S100" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2025; raw=2,523,000</t>
       </text>
     </comment>
-    <comment ref="N97" authorId="0" shapeId="0">
+    <comment ref="S101" authorId="0" shapeId="0">
       <text>
         <t>PropertyPlantAndEquipmentGross @ FY2025; raw=11,187,000</t>
       </text>
     </comment>
-    <comment ref="B104" authorId="0" shapeId="0">
+    <comment ref="B108" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ FY2024; raw=13,970,000</t>
       </text>
     </comment>
-    <comment ref="C104" authorId="0" shapeId="0">
+    <comment ref="C108" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ Q2 2025; raw=126,644,000</t>
       </text>
     </comment>
-    <comment ref="D104" authorId="0" shapeId="0">
+    <comment ref="D108" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ Q3 2025; raw=132,171,000</t>
       </text>
     </comment>
-    <comment ref="E104" authorId="0" shapeId="0">
+    <comment ref="E108" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ FY2025; raw=132,183,000</t>
       </text>
     </comment>
-    <comment ref="B105" authorId="0" shapeId="0">
+    <comment ref="F108" authorId="0" shapeId="0">
+      <text>
+        <t>FiniteLivedIntangibleAssetsGross @ Q1 2026; raw=131,865,000</t>
+      </text>
+    </comment>
+    <comment ref="B109" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ FY2024; raw=500,000</t>
       </text>
     </comment>
-    <comment ref="C105" authorId="0" shapeId="0">
+    <comment ref="C109" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ Q2 2025; raw=500,000</t>
       </text>
     </comment>
-    <comment ref="D105" authorId="0" shapeId="0">
+    <comment ref="D109" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ Q3 2025; raw=500,000</t>
       </text>
     </comment>
-    <comment ref="E105" authorId="0" shapeId="0">
+    <comment ref="E109" authorId="0" shapeId="0">
       <text>
         <t>FiniteLivedIntangibleAssetsGross @ FY2025; raw=500,000</t>
+      </text>
+    </comment>
+    <comment ref="F109" authorId="0" shapeId="0">
+      <text>
+        <t>FiniteLivedIntangibleAssetsGross @ Q1 2026; raw=500,000</t>
       </text>
     </comment>
   </commentList>
@@ -2052,7 +2394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R112"/>
+  <dimension ref="A1:W116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2153,6 +2495,11 @@
           <t>FY2025</t>
         </is>
       </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2197,6 +2544,9 @@
       <c r="K7" s="8" t="n">
         <v>2515269</v>
       </c>
+      <c r="L7" s="8" t="n">
+        <v>782615</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2241,6 +2591,9 @@
       <c r="K10" s="8" t="n">
         <v>125033</v>
       </c>
+      <c r="L10" s="8" t="n">
+        <v>137536</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2257,87 +2610,112 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2021</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Q2 2021</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Q3 2021</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
           <t>FY2021</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Q1 2022</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Q2 2022</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Q3 2022</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>FY2022</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>Q1 2023</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
         <is>
           <t>Q2 2023</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>Q3 2023</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>FY2023</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>Q1 2024</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="P15" s="5" t="inlineStr">
         <is>
           <t>Q2 2024</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>Q3 2024</t>
         </is>
       </c>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="R15" s="5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="O15" s="5" t="inlineStr">
+      <c r="S15" s="5" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="P15" s="5" t="inlineStr">
+      <c r="T15" s="5" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="Q15" s="5" t="inlineStr">
+      <c r="U15" s="5" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="R15" s="5" t="inlineStr">
+      <c r="V15" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
         </is>
       </c>
     </row>
@@ -2355,55 +2733,70 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>273005</v>
+        <v>95480.31</v>
       </c>
       <c r="C17" s="8" t="n">
+        <v>39003</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>53601</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>84490</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>273004.795</v>
+      </c>
+      <c r="G17" s="8" t="n">
         <v>123473</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="H17" s="8" t="n">
         <v>145409</v>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="I17" s="8" t="n">
         <v>179541</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="J17" s="8" t="n">
         <v>617457</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="K17" s="8" t="n">
         <v>248552</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="L17" s="8" t="n">
         <v>310815</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="M17" s="8" t="n">
         <v>371178</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="N17" s="8" t="n">
         <v>1263341</v>
       </c>
-      <c r="K17" s="8" t="n">
+      <c r="O17" s="8" t="n">
         <v>339512</v>
       </c>
-      <c r="L17" s="8" t="n">
+      <c r="P17" s="8" t="n">
         <v>382351</v>
       </c>
-      <c r="M17" s="8" t="n">
+      <c r="Q17" s="8" t="n">
         <v>247125</v>
       </c>
-      <c r="N17" s="8" t="n">
+      <c r="R17" s="8" t="n">
         <v>1280894</v>
       </c>
-      <c r="O17" s="8" t="n">
+      <c r="S17" s="8" t="n">
         <v>306534</v>
       </c>
-      <c r="P17" s="8" t="n">
+      <c r="T17" s="8" t="n">
         <v>714459</v>
       </c>
-      <c r="Q17" s="8" t="n">
+      <c r="U17" s="8" t="n">
         <v>701990</v>
       </c>
-      <c r="R17" s="8" t="n">
+      <c r="V17" s="8" t="n">
         <v>2422490</v>
+      </c>
+      <c r="W17" s="8" t="n">
+        <v>747316</v>
       </c>
     </row>
     <row r="18">
@@ -2413,55 +2806,70 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>38097</v>
+        <v>33727.441</v>
       </c>
       <c r="C18" s="8" t="n">
+        <v>10368</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>10792</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>9536</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>38097.016</v>
+      </c>
+      <c r="G18" s="8" t="n">
         <v>8495</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="H18" s="8" t="n">
         <v>7280</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="I18" s="8" t="n">
         <v>7546</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="J18" s="8" t="n">
         <v>31054</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="K18" s="8" t="n">
         <v>8652</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="L18" s="8" t="n">
         <v>11909</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="M18" s="8" t="n">
         <v>11038</v>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="N18" s="8" t="n">
         <v>43722</v>
       </c>
-      <c r="K18" s="8" t="n">
+      <c r="O18" s="8" t="n">
         <v>14142</v>
       </c>
-      <c r="L18" s="8" t="n">
+      <c r="P18" s="8" t="n">
         <v>16684</v>
       </c>
-      <c r="M18" s="8" t="n">
+      <c r="Q18" s="8" t="n">
         <v>16243</v>
       </c>
-      <c r="N18" s="8" t="n">
+      <c r="R18" s="8" t="n">
         <v>61696</v>
       </c>
-      <c r="O18" s="8" t="n">
+      <c r="S18" s="8" t="n">
         <v>18659</v>
       </c>
-      <c r="P18" s="8" t="n">
+      <c r="T18" s="8" t="n">
         <v>18301</v>
       </c>
-      <c r="Q18" s="8" t="n">
+      <c r="U18" s="8" t="n">
         <v>17691</v>
       </c>
-      <c r="R18" s="8" t="n">
+      <c r="V18" s="8" t="n">
         <v>72544</v>
+      </c>
+      <c r="W18" s="8" t="n">
+        <v>25354</v>
       </c>
     </row>
     <row r="19">
@@ -2471,39 +2879,51 @@
         </is>
       </c>
       <c r="B19" s="8" t="n">
+        <v>23400</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>7900</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F19" s="8" t="n">
         <v>26900</v>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="G19" s="8" t="n">
         <v>5800</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="H19" s="8" t="n">
         <v>5100</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="I19" s="8" t="n">
         <v>5300</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="J19" s="8" t="n">
         <v>21700</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="K19" s="8" t="n">
         <v>5500</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="L19" s="8" t="n">
         <v>7900</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="M19" s="8" t="n">
         <v>7400</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="N19" s="8" t="n">
         <v>29300</v>
       </c>
-      <c r="K19" s="8" t="n">
+      <c r="O19" s="8" t="n">
         <v>10000</v>
       </c>
-      <c r="L19" s="8" t="n">
+      <c r="P19" s="8" t="n">
         <v>11300</v>
       </c>
-      <c r="M19" s="8" t="n">
+      <c r="Q19" s="8" t="n">
         <v>9500</v>
       </c>
     </row>
@@ -2513,44 +2933,47 @@
           <t xml:space="preserve">  Asia Pacific</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="F20" s="8" t="n">
         <v>2538</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="J20" s="8" t="n">
         <v>3647</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="L20" s="8" t="n">
         <v>1606</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="M20" s="8" t="n">
         <v>1247</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="N20" s="8" t="n">
         <v>4755</v>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="O20" s="8" t="n">
         <v>675</v>
       </c>
-      <c r="L20" s="8" t="n">
+      <c r="P20" s="8" t="n">
         <v>860</v>
       </c>
-      <c r="M20" s="8" t="n">
+      <c r="Q20" s="8" t="n">
         <v>594</v>
       </c>
-      <c r="N20" s="8" t="n">
+      <c r="R20" s="8" t="n">
         <v>5658</v>
       </c>
-      <c r="O20" s="8" t="n">
+      <c r="S20" s="8" t="n">
         <v>2244</v>
       </c>
-      <c r="P20" s="8" t="n">
+      <c r="T20" s="8" t="n">
         <v>4381</v>
       </c>
-      <c r="Q20" s="8" t="n">
+      <c r="U20" s="8" t="n">
         <v>3518</v>
       </c>
-      <c r="R20" s="8" t="n">
+      <c r="V20" s="8" t="n">
         <v>12971</v>
+      </c>
+      <c r="W20" s="8" t="n">
+        <v>6995</v>
       </c>
     </row>
     <row r="21">
@@ -2560,55 +2983,70 @@
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>632</v>
+        <v>425.323</v>
       </c>
       <c r="C21" s="8" t="n">
+        <v>128</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>177</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>631.649</v>
+      </c>
+      <c r="G21" s="8" t="n">
         <v>454</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="H21" s="8" t="n">
         <v>448</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="I21" s="8" t="n">
         <v>182</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="J21" s="8" t="n">
         <v>1446</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="K21" s="8" t="n">
         <v>1477</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="L21" s="8" t="n">
         <v>1553</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="M21" s="8" t="n">
         <v>1294</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="N21" s="8" t="n">
         <v>6196</v>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="O21" s="8" t="n">
         <v>1379</v>
       </c>
-      <c r="L21" s="8" t="n">
+      <c r="P21" s="8" t="n">
         <v>2082</v>
       </c>
-      <c r="M21" s="8" t="n">
+      <c r="Q21" s="8" t="n">
         <v>1786</v>
       </c>
-      <c r="N21" s="8" t="n">
+      <c r="R21" s="8" t="n">
         <v>7382</v>
       </c>
-      <c r="O21" s="8" t="n">
+      <c r="S21" s="8" t="n">
         <v>1839</v>
       </c>
-      <c r="P21" s="8" t="n">
+      <c r="T21" s="8" t="n">
         <v>2118</v>
       </c>
-      <c r="Q21" s="8" t="n">
+      <c r="U21" s="8" t="n">
         <v>1907</v>
       </c>
-      <c r="R21" s="8" t="n">
+      <c r="V21" s="8" t="n">
         <v>7264</v>
+      </c>
+      <c r="W21" s="8" t="n">
+        <v>2950</v>
       </c>
     </row>
     <row r="22">
@@ -2617,25 +3055,43 @@
           <t xml:space="preserve">  Asia</t>
         </is>
       </c>
+      <c r="B22" s="8" t="n">
+        <v>1092.703</v>
+      </c>
       <c r="C22" s="8" t="n">
+        <v>536</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>619</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>706</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>2538.099</v>
+      </c>
+      <c r="G22" s="8" t="n">
         <v>966</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="H22" s="8" t="n">
         <v>883</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="I22" s="8" t="n">
         <v>964</v>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="J22" s="8" t="n">
+        <v>3647</v>
+      </c>
+      <c r="K22" s="8" t="n">
         <v>1258</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="L22" s="8" t="n">
         <v>1606</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="M22" s="8" t="n">
         <v>1247</v>
       </c>
-      <c r="K22" s="8" t="n">
+      <c r="O22" s="8" t="n">
         <v>675</v>
       </c>
     </row>
@@ -2652,29 +3108,32 @@
           <t xml:space="preserve">  North America</t>
         </is>
       </c>
-      <c r="J25" s="8" t="n">
+      <c r="N25" s="8" t="n">
         <v>24316</v>
       </c>
-      <c r="L25" s="8" t="n">
+      <c r="P25" s="8" t="n">
         <v>34894</v>
       </c>
-      <c r="M25" s="8" t="n">
+      <c r="Q25" s="8" t="n">
         <v>37023</v>
       </c>
-      <c r="N25" s="8" t="n">
+      <c r="R25" s="8" t="n">
         <v>72115</v>
       </c>
-      <c r="O25" s="8" t="n">
+      <c r="S25" s="8" t="n">
         <v>73023</v>
       </c>
-      <c r="P25" s="8" t="n">
+      <c r="T25" s="8" t="n">
         <v>190854</v>
       </c>
-      <c r="Q25" s="8" t="n">
+      <c r="U25" s="8" t="n">
         <v>197635</v>
       </c>
-      <c r="R25" s="8" t="n">
+      <c r="V25" s="8" t="n">
         <v>197866</v>
+      </c>
+      <c r="W25" s="8" t="n">
+        <v>202300</v>
       </c>
     </row>
     <row r="26">
@@ -2683,28 +3142,28 @@
           <t xml:space="preserve">  Sweden</t>
         </is>
       </c>
-      <c r="J26" s="8" t="n">
+      <c r="N26" s="8" t="n">
         <v>2212</v>
       </c>
-      <c r="L26" s="8" t="n">
+      <c r="P26" s="8" t="n">
         <v>2550</v>
       </c>
-      <c r="M26" s="8" t="n">
+      <c r="Q26" s="8" t="n">
         <v>2663</v>
       </c>
-      <c r="N26" s="8" t="n">
+      <c r="R26" s="8" t="n">
         <v>2523</v>
       </c>
-      <c r="O26" s="8" t="n">
+      <c r="S26" s="8" t="n">
         <v>3744</v>
       </c>
-      <c r="P26" s="8" t="n">
+      <c r="T26" s="8" t="n">
         <v>4057</v>
       </c>
-      <c r="Q26" s="8" t="n">
+      <c r="U26" s="8" t="n">
         <v>4441</v>
       </c>
-      <c r="R26" s="8" t="n">
+      <c r="V26" s="8" t="n">
         <v>4635</v>
       </c>
     </row>
@@ -2714,19 +3173,19 @@
           <t xml:space="preserve">  Foreign Ops (ex-IE/SE/FI)</t>
         </is>
       </c>
-      <c r="N27" s="8" t="n">
+      <c r="R27" s="8" t="n">
         <v>17101</v>
       </c>
-      <c r="O27" s="8" t="n">
+      <c r="S27" s="8" t="n">
         <v>18708</v>
       </c>
-      <c r="P27" s="8" t="n">
+      <c r="T27" s="8" t="n">
         <v>19759</v>
       </c>
-      <c r="Q27" s="8" t="n">
+      <c r="U27" s="8" t="n">
         <v>20201</v>
       </c>
-      <c r="R27" s="8" t="n">
+      <c r="V27" s="8" t="n">
         <v>20263</v>
       </c>
     </row>
@@ -2736,28 +3195,28 @@
           <t xml:space="preserve">  Finland</t>
         </is>
       </c>
-      <c r="J28" s="8" t="n">
+      <c r="N28" s="8" t="n">
         <v>12153</v>
       </c>
-      <c r="L28" s="8" t="n">
+      <c r="P28" s="8" t="n">
         <v>11591</v>
       </c>
-      <c r="M28" s="8" t="n">
+      <c r="Q28" s="8" t="n">
         <v>11930</v>
       </c>
-      <c r="N28" s="8" t="n">
+      <c r="R28" s="8" t="n">
         <v>10950</v>
       </c>
-      <c r="O28" s="8" t="n">
+      <c r="S28" s="8" t="n">
         <v>11261</v>
       </c>
-      <c r="P28" s="8" t="n">
+      <c r="T28" s="8" t="n">
         <v>12030</v>
       </c>
-      <c r="Q28" s="8" t="n">
+      <c r="U28" s="8" t="n">
         <v>12133</v>
       </c>
-      <c r="R28" s="8" t="n">
+      <c r="V28" s="8" t="n">
         <v>12004</v>
       </c>
     </row>
@@ -2767,16 +3226,16 @@
           <t xml:space="preserve">  International (ex-NA)</t>
         </is>
       </c>
-      <c r="J29" s="8" t="n">
+      <c r="N29" s="8" t="n">
         <v>14394</v>
       </c>
-      <c r="L29" s="8" t="n">
+      <c r="P29" s="8" t="n">
         <v>14171</v>
       </c>
-      <c r="M29" s="8" t="n">
+      <c r="Q29" s="8" t="n">
         <v>18477</v>
       </c>
-      <c r="N29" s="8" t="n">
+      <c r="R29" s="8" t="n">
         <v>17101</v>
       </c>
     </row>
@@ -2786,709 +3245,751 @@
           <t xml:space="preserve">  Other (geography)</t>
         </is>
       </c>
-      <c r="J30" s="8" t="n">
-        <v>29</v>
-      </c>
-      <c r="L30" s="8" t="n">
-        <v>30</v>
-      </c>
-      <c r="M30" s="8" t="n">
-        <v>30</v>
-      </c>
       <c r="N30" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="O30" s="8" t="n">
+      <c r="P30" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="P30" s="8" t="n">
-        <v>29</v>
-      </c>
       <c r="Q30" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R30" s="8" t="n">
         <v>29</v>
       </c>
+      <c r="S30" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="T30" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="U30" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="V30" s="8" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  celh:GeographicalNonNorthAmericaMember</t>
+        </is>
+      </c>
+      <c r="V31" s="8" t="n">
+        <v>20300</v>
+      </c>
+      <c r="W31" s="8" t="n">
+        <v>21100</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Ireland</t>
         </is>
       </c>
-      <c r="M31" s="8" t="n">
+      <c r="Q32" s="8" t="n">
         <v>3854</v>
       </c>
-      <c r="N31" s="8" t="n">
+      <c r="R32" s="8" t="n">
         <v>3599</v>
       </c>
-      <c r="O31" s="8" t="n">
+      <c r="S32" s="8" t="n">
         <v>3673</v>
       </c>
-      <c r="P31" s="8" t="n">
+      <c r="T32" s="8" t="n">
         <v>3643</v>
       </c>
-      <c r="Q31" s="8" t="n">
+      <c r="U32" s="8" t="n">
         <v>3598</v>
       </c>
-      <c r="R31" s="8" t="n">
+      <c r="V32" s="8" t="n">
         <v>3595</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>25. CUSTOMER CONCENTRATION (% OF REVENUE)  (% of revenue)</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>25. CUSTOMER CONCENTRATION (% OF REVENUE)  (% values)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Metric / Segment</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Q1 2022</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Q2 2022</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Q3 2022</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>FY2022</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>Q1 2023</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Q2 2023</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>Q3 2023</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>FY2023</t>
         </is>
       </c>
-      <c r="J36" s="5" t="inlineStr">
+      <c r="J37" s="5" t="inlineStr">
         <is>
           <t>Q1 2024</t>
         </is>
       </c>
-      <c r="K36" s="5" t="inlineStr">
+      <c r="K37" s="5" t="inlineStr">
         <is>
           <t>Q2 2024</t>
         </is>
       </c>
-      <c r="L36" s="5" t="inlineStr">
+      <c r="L37" s="5" t="inlineStr">
         <is>
           <t>Q3 2024</t>
         </is>
       </c>
-      <c r="M36" s="5" t="inlineStr">
+      <c r="M37" s="5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="N36" s="5" t="inlineStr">
+      <c r="N37" s="5" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="O36" s="5" t="inlineStr">
+      <c r="O37" s="5" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="P36" s="5" t="inlineStr">
+      <c r="P37" s="5" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="Q36" s="5" t="inlineStr">
+      <c r="Q37" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>% of Revenue</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PepsiCo Inc.</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="n">
-        <v>0.476</v>
-      </c>
-      <c r="D38" s="9" t="n">
-        <v>0.312</v>
-      </c>
-      <c r="E38" s="9" t="n">
-        <v>0.476</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>0.6020000000000001</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <v>0.5670000000000001</v>
-      </c>
-      <c r="H38" s="9" t="n">
-        <v>0.6459999999999999</v>
-      </c>
-      <c r="I38" s="9" t="n">
-        <v>0.594</v>
-      </c>
-      <c r="J38" s="9" t="n">
-        <v>0.5920000000000001</v>
-      </c>
-      <c r="K38" s="9" t="n">
-        <v>0.529</v>
-      </c>
-      <c r="L38" s="9" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="M38" s="9" t="n">
-        <v>0.547</v>
-      </c>
-      <c r="N38" s="9" t="n">
-        <v>0.5760000000000001</v>
-      </c>
-      <c r="O38" s="9" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="P38" s="9" t="n">
-        <v>0.354</v>
-      </c>
-      <c r="Q38" s="9" t="n">
-        <v>0.4320000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  All Other</t>
+          <t xml:space="preserve">  PepsiCo Inc.</t>
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>0.7220000000000001</v>
-      </c>
-      <c r="C39" s="9" t="n">
-        <v>0.841</v>
+        <v>0.476</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.312</v>
       </c>
       <c r="E39" s="9" t="n">
-        <v>0.406</v>
+        <v>0.476</v>
       </c>
       <c r="F39" s="9" t="n">
-        <v>0.185</v>
+        <v>0.6020000000000001</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>0.303</v>
+        <v>0.5670000000000001</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.265</v>
+        <v>0.6459999999999999</v>
       </c>
       <c r="I39" s="9" t="n">
-        <v>0.286</v>
+        <v>0.594</v>
       </c>
       <c r="J39" s="9" t="n">
-        <v>0.306</v>
+        <v>0.5920000000000001</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>0.35</v>
+        <v>0.529</v>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.279</v>
+        <v>0.47</v>
       </c>
       <c r="M39" s="9" t="n">
-        <v>0.337</v>
+        <v>0.547</v>
       </c>
       <c r="N39" s="9" t="n">
-        <v>0.244</v>
+        <v>0.5760000000000001</v>
       </c>
       <c r="O39" s="9" t="n">
-        <v>0.55</v>
+        <v>0.333</v>
       </c>
       <c r="P39" s="9" t="n">
-        <v>0.48</v>
+        <v>0.354</v>
       </c>
       <c r="Q39" s="9" t="n">
-        <v>0.46</v>
+        <v>0.4320000000000001</v>
+      </c>
+      <c r="R39" s="9" t="n">
+        <v>0.59</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Costco</t>
+          <t xml:space="preserve">  All Other</t>
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>0.175</v>
+        <v>0.7220000000000001</v>
       </c>
       <c r="C40" s="9" t="n">
-        <v>0.159</v>
+        <v>0.841</v>
       </c>
       <c r="D40" s="9" t="n">
-        <v>0.129</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="E40" s="9" t="n">
-        <v>0.167</v>
+        <v>0.406</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>0.129</v>
+        <v>0.185</v>
       </c>
       <c r="G40" s="9" t="n">
-        <v>0.13</v>
+        <v>0.303</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.08900000000000001</v>
+        <v>0.265</v>
       </c>
       <c r="I40" s="9" t="n">
-        <v>0.12</v>
+        <v>0.286</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>0.102</v>
+        <v>0.306</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>0.121</v>
+        <v>0.35</v>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.149</v>
+        <v>0.279</v>
       </c>
       <c r="M40" s="9" t="n">
-        <v>0.116</v>
+        <v>0.337</v>
       </c>
       <c r="N40" s="9" t="n">
-        <v>0.059</v>
+        <v>0.244</v>
       </c>
       <c r="O40" s="9" t="n">
-        <v>0.117</v>
+        <v>0.55</v>
       </c>
       <c r="P40" s="9" t="n">
-        <v>0.111</v>
+        <v>0.48</v>
       </c>
       <c r="Q40" s="9" t="n">
-        <v>0.108</v>
+        <v>0.46</v>
+      </c>
+      <c r="R40" s="9" t="n">
+        <v>0.326</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Costco</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="D41" s="9" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>0.08900000000000001</v>
+      </c>
+      <c r="I41" s="9" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="K41" s="9" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="L41" s="9" t="n">
+        <v>0.149</v>
+      </c>
+      <c r="M41" s="9" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="N41" s="9" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="O41" s="9" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="P41" s="9" t="n">
+        <v>0.111</v>
+      </c>
+      <c r="Q41" s="9" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="R41" s="9" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Amazon</t>
         </is>
       </c>
-      <c r="B41" s="9" t="n">
+      <c r="B42" s="9" t="n">
         <v>0.103</v>
       </c>
-      <c r="E41" s="9" t="n">
+      <c r="E42" s="9" t="n">
         <v>0.118</v>
       </c>
-      <c r="F41" s="9" t="n">
+      <c r="F42" s="9" t="n">
         <v>0.08400000000000001</v>
       </c>
-      <c r="H41" s="9" t="n">
+      <c r="H42" s="9" t="n">
         <v>0.058</v>
       </c>
-      <c r="I41" s="9" t="n">
+      <c r="I42" s="9" t="n">
         <v>0.059</v>
       </c>
-      <c r="J41" s="9" t="n">
+      <c r="J42" s="9" t="n">
         <v>0.08</v>
       </c>
-      <c r="L41" s="9" t="n">
+      <c r="L42" s="9" t="n">
         <v>0.102</v>
       </c>
-      <c r="M41" s="9" t="n">
+      <c r="M42" s="9" t="n">
         <v>0.08900000000000001</v>
       </c>
-      <c r="N41" s="9" t="n">
+      <c r="N42" s="9" t="n">
         <v>0.121</v>
       </c>
-      <c r="P41" s="9" t="n">
+      <c r="P42" s="9" t="n">
         <v>0.055</v>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="R42" s="9" t="n">
+        <v>0.08400000000000001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>3. M&amp;A PRO FORMA + ACQUISITION CONTRIBUTION  ($ in thousands)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Metric / Segment</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Q2 2024</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>Q3 2024</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr">
+      <c r="H47" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
         </is>
       </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Pro Forma Revenue</t>
         </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Alani Nu + Rockstar (combined)</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="n">
-        <v>513912</v>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>2317965</v>
-      </c>
-      <c r="G48" s="8" t="n">
-        <v>798496</v>
-      </c>
-      <c r="H48" s="8" t="n">
-        <v>3003677</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Alani Nu + Rockstar (combined)</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>513912</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>2317965</v>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>647397</v>
+      </c>
+      <c r="G49" s="8" t="n">
+        <v>798496</v>
+      </c>
+      <c r="H49" s="8" t="n">
+        <v>3003677</v>
+      </c>
+      <c r="I49" s="8" t="n">
+        <v>782615</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Alani Nu</t>
         </is>
       </c>
-      <c r="B49" s="8" t="n">
+      <c r="B50" s="8" t="n">
         <v>547650</v>
       </c>
-      <c r="F49" s="8" t="n">
+      <c r="F50" s="8" t="n">
         <v>739259</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Pro Forma Net Income</t>
         </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Alani Nu + Rockstar (combined)</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="n">
-        <v>17015</v>
-      </c>
-      <c r="D52" s="8" t="n">
-        <v>147638</v>
-      </c>
-      <c r="G52" s="8" t="n">
-        <v>-51019</v>
-      </c>
-      <c r="H52" s="8" t="n">
-        <v>218748</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Alani Nu + Rockstar (combined)</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="n">
+        <v>17015</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>147638</v>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>98690</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>-51019</v>
+      </c>
+      <c r="H53" s="8" t="n">
+        <v>218748</v>
+      </c>
+      <c r="I53" s="8" t="n">
+        <v>110099</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Alani Nu</t>
         </is>
       </c>
-      <c r="B53" s="8" t="n">
+      <c r="B54" s="8" t="n">
         <v>70659</v>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F54" s="8" t="n">
         <v>116424</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Purchase Price</t>
         </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Alani Nu</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="n">
-        <v>1775000</v>
-      </c>
-      <c r="F56" s="8" t="n">
-        <v>2055589</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Alani Nu</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="n">
+        <v>1775000</v>
+      </c>
+      <c r="F57" s="8" t="n">
+        <v>2055589</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Rockstar</t>
         </is>
       </c>
-      <c r="G57" s="8" t="n">
+      <c r="G58" s="8" t="n">
         <v>307603</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>4. DEBT SCHEDULE  ($ in thousands)</t>
-        </is>
-      </c>
-    </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>4. DEBT SCHEDULE  (mixed: $ in thousands, % / counts as labeled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>Metric / Segment</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Q4 2025</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E63" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
         </is>
       </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="inlineStr">
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>Carrying Amount</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="7" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  Term Loan Facility</t>
         </is>
       </c>
-      <c r="D64" s="8" t="n">
+      <c r="D65" s="8" t="n">
         <v>700000</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="6" t="inlineStr">
-        <is>
-          <t>Effective Rate (raw decimal)</t>
-        </is>
-      </c>
-    </row>
     <row r="67">
-      <c r="A67" s="7" t="inlineStr">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>Effective Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  Term Loan Facility</t>
         </is>
       </c>
-      <c r="B67" s="8" t="n">
-        <v>8.16e-05</v>
-      </c>
-      <c r="C67" s="8" t="n">
-        <v>7.9e-05</v>
-      </c>
-      <c r="E67" s="8" t="n">
-        <v>7.09e-05</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>5. STOCK-BASED COMPENSATION BY AWARD TYPE  ($ in thousands)</t>
-        </is>
+      <c r="B68" s="9" t="n">
+        <v>0.08160000000000001</v>
+      </c>
+      <c r="C68" s="9" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>0.0709</v>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>0.0678</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>5. STOCK-BASED COMPENSATION BY AWARD TYPE  (mixed: $ in thousands, % / counts as labeled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>Metric / Segment</t>
         </is>
       </c>
-      <c r="B72" s="5" t="inlineStr">
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2021</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>FY2021</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>Q1 2022</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="F73" s="5" t="inlineStr">
         <is>
           <t>FY2022</t>
         </is>
       </c>
-      <c r="E72" s="5" t="inlineStr">
+      <c r="G73" s="5" t="inlineStr">
         <is>
           <t>Q1 2023</t>
         </is>
       </c>
-      <c r="F72" s="5" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>FY2023</t>
         </is>
       </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>Q1 2024</t>
         </is>
       </c>
-      <c r="H72" s="5" t="inlineStr">
+      <c r="J73" s="5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="I72" s="5" t="inlineStr">
+      <c r="K73" s="5" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="J72" s="5" t="inlineStr">
+      <c r="L73" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
         </is>
       </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>Wtd Avg Grant FV $</t>
+      <c r="M73" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RSUs</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="n">
-        <v>0.02471</v>
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>Wtd Avg Grant FV (per share)</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  RSUs</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="n">
+        <v>24.71</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  PSUs</t>
         </is>
       </c>
-      <c r="D75" s="8" t="n">
-        <v>0.02155</v>
-      </c>
-      <c r="F75" s="8" t="n">
-        <v>0.03276</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="6" t="inlineStr">
+      <c r="F76" s="10" t="n">
+        <v>21.55</v>
+      </c>
+      <c r="H76" s="10" t="n">
+        <v>32.76</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>Shares Granted #</t>
         </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RSUs</t>
-        </is>
-      </c>
-      <c r="B78" s="8" t="n">
-        <v>1700</v>
-      </c>
-      <c r="C78" s="8" t="n">
-        <v>189</v>
-      </c>
-      <c r="D78" s="8" t="n">
-        <v>700</v>
-      </c>
-      <c r="E78" s="8" t="n">
-        <v>124</v>
-      </c>
-      <c r="F78" s="8" t="n">
-        <v>468</v>
-      </c>
-      <c r="G78" s="8" t="n">
-        <v>210</v>
-      </c>
-      <c r="H78" s="8" t="n">
-        <v>377</v>
       </c>
     </row>
     <row r="79">
@@ -3497,478 +3998,641 @@
           <t xml:space="preserve">  RSUs + PSUs (combined)</t>
         </is>
       </c>
-      <c r="G79" s="8" t="n">
-        <v>275</v>
-      </c>
-      <c r="H79" s="8" t="n">
-        <v>552</v>
-      </c>
       <c r="I79" s="8" t="n">
-        <v>1074</v>
+        <v>275000</v>
       </c>
       <c r="J79" s="8" t="n">
-        <v>1628</v>
+        <v>552000</v>
+      </c>
+      <c r="K79" s="8" t="n">
+        <v>1074000</v>
+      </c>
+      <c r="L79" s="8" t="n">
+        <v>1628000</v>
+      </c>
+      <c r="M79" s="8" t="n">
+        <v>805000</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  RSUs</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="n">
+        <v>468000</v>
+      </c>
+      <c r="D80" s="8" t="n">
+        <v>573428</v>
+      </c>
+      <c r="E80" s="8" t="n">
+        <v>189000</v>
+      </c>
+      <c r="F80" s="8" t="n">
+        <v>248</v>
+      </c>
+      <c r="G80" s="8" t="n">
+        <v>124000</v>
+      </c>
+      <c r="H80" s="8" t="n">
+        <v>468000</v>
+      </c>
+      <c r="I80" s="8" t="n">
+        <v>210000</v>
+      </c>
+      <c r="J80" s="8" t="n">
+        <v>377000</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  PSUs</t>
         </is>
       </c>
-      <c r="B80" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="D80" s="8" t="n">
-        <v>228</v>
-      </c>
-      <c r="G80" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="H80" s="8" t="n">
-        <v>175</v>
-      </c>
-      <c r="I80" s="8" t="n">
-        <v>142</v>
-      </c>
-      <c r="J80" s="8" t="n">
-        <v>142</v>
+      <c r="D81" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F81" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="I81" s="8" t="n">
+        <v>65000</v>
+      </c>
+      <c r="J81" s="8" t="n">
+        <v>175000</v>
+      </c>
+      <c r="K81" s="8" t="n">
+        <v>142000</v>
+      </c>
+      <c r="L81" s="8" t="n">
+        <v>142000</v>
+      </c>
+      <c r="M81" s="8" t="n">
+        <v>67000</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
-        <is>
-          <t>Shares Vested #</t>
-        </is>
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  us-gaap:RestrictedStockMember</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="n">
+        <v>175737</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  celh:StockBasedAwardsIssuedToNonEmployeeConsultantsMember</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n">
+        <v>15468</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>Shares Vested #</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RSUs + PSUs (combined)</t>
+        </is>
+      </c>
+      <c r="I86" s="8" t="n">
+        <v>510000</v>
+      </c>
+      <c r="J86" s="8" t="n">
+        <v>803000</v>
+      </c>
+      <c r="K86" s="8" t="n">
+        <v>249000</v>
+      </c>
+      <c r="L86" s="8" t="n">
+        <v>470000</v>
+      </c>
+      <c r="M86" s="8" t="n">
+        <v>478000</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  RSUs</t>
         </is>
       </c>
-      <c r="C83" s="8" t="n">
-        <v>111</v>
-      </c>
-      <c r="E83" s="8" t="n">
-        <v>157</v>
-      </c>
-      <c r="F83" s="8" t="n">
-        <v>670</v>
-      </c>
-      <c r="G83" s="8" t="n">
-        <v>510</v>
-      </c>
-      <c r="H83" s="8" t="n">
-        <v>715</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  RSUs + PSUs (combined)</t>
-        </is>
-      </c>
-      <c r="G84" s="8" t="n">
-        <v>510</v>
-      </c>
-      <c r="H84" s="8" t="n">
-        <v>803</v>
-      </c>
-      <c r="I84" s="8" t="n">
-        <v>249</v>
-      </c>
-      <c r="J84" s="8" t="n">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="7" t="inlineStr">
+      <c r="D87" s="8" t="n">
+        <v>18758</v>
+      </c>
+      <c r="E87" s="8" t="n">
+        <v>111000</v>
+      </c>
+      <c r="F87" s="8" t="n">
+        <v>205</v>
+      </c>
+      <c r="G87" s="8" t="n">
+        <v>157000</v>
+      </c>
+      <c r="H87" s="8" t="n">
+        <v>670000</v>
+      </c>
+      <c r="I87" s="8" t="n">
+        <v>510000</v>
+      </c>
+      <c r="J87" s="8" t="n">
+        <v>715000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  PSUs</t>
         </is>
       </c>
-      <c r="F85" s="8" t="n">
-        <v>92</v>
-      </c>
-      <c r="H85" s="8" t="n">
-        <v>78</v>
+      <c r="F88" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="H88" s="8" t="n">
+        <v>92000</v>
+      </c>
+      <c r="J88" s="8" t="n">
+        <v>78000</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>7. PP&amp;E BY CLASS  ($ in thousands)</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="4" t="inlineStr">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  us-gaap:RestrictedStockMember</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="n">
+        <v>170145</v>
+      </c>
+      <c r="D89" s="8" t="n">
+        <v>18913</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>7. PP&amp;E BY CLASS  (mixed: $ in thousands, % / counts as labeled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>Metric / Segment</t>
         </is>
       </c>
-      <c r="B90" s="5" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2022</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Q2 2022</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Q3 2022</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
         <is>
           <t>FY2022</t>
         </is>
       </c>
-      <c r="C90" s="5" t="inlineStr">
+      <c r="H94" s="5" t="inlineStr">
         <is>
           <t>Q1 2023</t>
         </is>
       </c>
-      <c r="D90" s="5" t="inlineStr">
+      <c r="I94" s="5" t="inlineStr">
         <is>
           <t>Q2 2023</t>
         </is>
       </c>
-      <c r="E90" s="5" t="inlineStr">
+      <c r="J94" s="5" t="inlineStr">
         <is>
           <t>Q3 2023</t>
         </is>
       </c>
-      <c r="F90" s="5" t="inlineStr">
+      <c r="K94" s="5" t="inlineStr">
         <is>
           <t>FY2023</t>
         </is>
       </c>
-      <c r="G90" s="5" t="inlineStr">
+      <c r="L94" s="5" t="inlineStr">
         <is>
           <t>Q1 2024</t>
         </is>
       </c>
-      <c r="H90" s="5" t="inlineStr">
+      <c r="M94" s="5" t="inlineStr">
         <is>
           <t>Q2 2024</t>
         </is>
       </c>
-      <c r="I90" s="5" t="inlineStr">
+      <c r="N94" s="5" t="inlineStr">
         <is>
           <t>Q3 2024</t>
         </is>
       </c>
-      <c r="J90" s="5" t="inlineStr">
+      <c r="O94" s="5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="K90" s="5" t="inlineStr">
+      <c r="P94" s="5" t="inlineStr">
         <is>
           <t>Q1 2025</t>
         </is>
       </c>
-      <c r="L90" s="5" t="inlineStr">
+      <c r="Q94" s="5" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="M90" s="5" t="inlineStr">
+      <c r="R94" s="5" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="N90" s="5" t="inlineStr">
+      <c r="S94" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="6" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
         <is>
           <t>Gross PP&amp;E</t>
         </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Merchandising Equipment / Coolers</t>
-        </is>
-      </c>
-      <c r="B92" s="8" t="n">
-        <v>9885</v>
-      </c>
-      <c r="C92" s="8" t="n">
-        <v>11848</v>
-      </c>
-      <c r="D92" s="8" t="n">
-        <v>14962</v>
-      </c>
-      <c r="E92" s="8" t="n">
-        <v>18703</v>
-      </c>
-      <c r="F92" s="8" t="n">
-        <v>21908</v>
-      </c>
-      <c r="G92" s="8" t="n">
-        <v>26110</v>
-      </c>
-      <c r="H92" s="8" t="n">
-        <v>34844</v>
-      </c>
-      <c r="I92" s="8" t="n">
-        <v>36573</v>
-      </c>
-      <c r="J92" s="8" t="n">
-        <v>39231</v>
-      </c>
-      <c r="K92" s="8" t="n">
-        <v>43441</v>
-      </c>
-      <c r="L92" s="8" t="n">
-        <v>52892</v>
-      </c>
-      <c r="M92" s="8" t="n">
-        <v>57158</v>
-      </c>
-      <c r="N92" s="8" t="n">
-        <v>60615</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Vehicles</t>
-        </is>
-      </c>
-      <c r="B93" s="8" t="n">
-        <v>1257</v>
-      </c>
-      <c r="C93" s="8" t="n">
-        <v>1524</v>
-      </c>
-      <c r="D93" s="8" t="n">
-        <v>2596</v>
-      </c>
-      <c r="E93" s="8" t="n">
-        <v>4617</v>
-      </c>
-      <c r="F93" s="8" t="n">
-        <v>6143</v>
-      </c>
-      <c r="G93" s="8" t="n">
-        <v>6294</v>
-      </c>
-      <c r="H93" s="8" t="n">
-        <v>6687</v>
-      </c>
-      <c r="I93" s="8" t="n">
-        <v>9070</v>
-      </c>
-      <c r="J93" s="8" t="n">
-        <v>12237</v>
-      </c>
-      <c r="K93" s="8" t="n">
-        <v>12237</v>
-      </c>
-      <c r="L93" s="8" t="n">
-        <v>14828</v>
-      </c>
-      <c r="M93" s="8" t="n">
-        <v>14919</v>
-      </c>
-      <c r="N93" s="8" t="n">
-        <v>17501</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Machinery &amp; Equipment</t>
-        </is>
-      </c>
-      <c r="J94" s="8" t="n">
-        <v>10136</v>
-      </c>
-      <c r="K94" s="8" t="n">
-        <v>11683</v>
-      </c>
-      <c r="L94" s="8" t="n">
-        <v>16585</v>
-      </c>
-      <c r="M94" s="8" t="n">
-        <v>22430</v>
-      </c>
-      <c r="N94" s="8" t="n">
-        <v>14631</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Office Equipment</t>
-        </is>
-      </c>
-      <c r="B95" s="8" t="n">
-        <v>1124</v>
-      </c>
-      <c r="C95" s="8" t="n">
-        <v>1158</v>
-      </c>
-      <c r="D95" s="8" t="n">
-        <v>1286</v>
-      </c>
-      <c r="E95" s="8" t="n">
-        <v>1399</v>
-      </c>
-      <c r="F95" s="8" t="n">
-        <v>1467</v>
-      </c>
-      <c r="G95" s="8" t="n">
-        <v>1571</v>
-      </c>
-      <c r="H95" s="8" t="n">
-        <v>1623</v>
-      </c>
-      <c r="I95" s="8" t="n">
-        <v>1632</v>
-      </c>
-      <c r="J95" s="8" t="n">
-        <v>2228</v>
-      </c>
-      <c r="K95" s="8" t="n">
-        <v>1681</v>
-      </c>
-      <c r="L95" s="8" t="n">
-        <v>1846</v>
-      </c>
-      <c r="M95" s="8" t="n">
-        <v>2880</v>
-      </c>
-      <c r="N95" s="8" t="n">
-        <v>3570</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Leasehold Improvements</t>
-        </is>
+          <t xml:space="preserve">  Merchandising Equipment / Coolers</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="n">
+        <v>394.418</v>
+      </c>
+      <c r="C96" s="8" t="n">
+        <v>3051.938</v>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>3561</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>4944</v>
+      </c>
+      <c r="F96" s="8" t="n">
+        <v>5505</v>
+      </c>
+      <c r="G96" s="8" t="n">
+        <v>9885</v>
+      </c>
+      <c r="H96" s="8" t="n">
+        <v>11848</v>
+      </c>
+      <c r="I96" s="8" t="n">
+        <v>14962</v>
       </c>
       <c r="J96" s="8" t="n">
-        <v>2561</v>
+        <v>18703</v>
       </c>
       <c r="K96" s="8" t="n">
-        <v>2375</v>
+        <v>21908</v>
       </c>
       <c r="L96" s="8" t="n">
-        <v>2439</v>
+        <v>26110</v>
       </c>
       <c r="M96" s="8" t="n">
-        <v>2443</v>
+        <v>34844</v>
       </c>
       <c r="N96" s="8" t="n">
-        <v>2523</v>
+        <v>36573</v>
+      </c>
+      <c r="O96" s="8" t="n">
+        <v>39231</v>
+      </c>
+      <c r="P96" s="8" t="n">
+        <v>43441</v>
+      </c>
+      <c r="Q96" s="8" t="n">
+        <v>52892</v>
+      </c>
+      <c r="R96" s="8" t="n">
+        <v>57158</v>
+      </c>
+      <c r="S96" s="8" t="n">
+        <v>60615</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Vehicles</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="n">
+        <v>78.124</v>
+      </c>
+      <c r="C97" s="8" t="n">
+        <v>304.21</v>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>456</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>739</v>
+      </c>
+      <c r="F97" s="8" t="n">
+        <v>1013</v>
+      </c>
+      <c r="G97" s="8" t="n">
+        <v>1257</v>
+      </c>
+      <c r="H97" s="8" t="n">
+        <v>1524</v>
+      </c>
+      <c r="I97" s="8" t="n">
+        <v>2596</v>
+      </c>
+      <c r="J97" s="8" t="n">
+        <v>4617</v>
+      </c>
+      <c r="K97" s="8" t="n">
+        <v>6143</v>
+      </c>
+      <c r="L97" s="8" t="n">
+        <v>6294</v>
+      </c>
+      <c r="M97" s="8" t="n">
+        <v>6687</v>
+      </c>
+      <c r="N97" s="8" t="n">
+        <v>9070</v>
+      </c>
+      <c r="O97" s="8" t="n">
+        <v>12237</v>
+      </c>
+      <c r="P97" s="8" t="n">
+        <v>12237</v>
+      </c>
+      <c r="Q97" s="8" t="n">
+        <v>14828</v>
+      </c>
+      <c r="R97" s="8" t="n">
+        <v>14919</v>
+      </c>
+      <c r="S97" s="8" t="n">
+        <v>17501</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Machinery &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="O98" s="8" t="n">
+        <v>10136</v>
+      </c>
+      <c r="P98" s="8" t="n">
+        <v>11683</v>
+      </c>
+      <c r="Q98" s="8" t="n">
+        <v>16585</v>
+      </c>
+      <c r="R98" s="8" t="n">
+        <v>22430</v>
+      </c>
+      <c r="S98" s="8" t="n">
+        <v>14631</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Office Equipment</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="n">
+        <v>630.759</v>
+      </c>
+      <c r="C99" s="8" t="n">
+        <v>890.6950000000001</v>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>968</v>
+      </c>
+      <c r="E99" s="8" t="n">
+        <v>996</v>
+      </c>
+      <c r="F99" s="8" t="n">
+        <v>1177</v>
+      </c>
+      <c r="G99" s="8" t="n">
+        <v>1124</v>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>1158</v>
+      </c>
+      <c r="I99" s="8" t="n">
+        <v>1286</v>
+      </c>
+      <c r="J99" s="8" t="n">
+        <v>1399</v>
+      </c>
+      <c r="K99" s="8" t="n">
+        <v>1467</v>
+      </c>
+      <c r="L99" s="8" t="n">
+        <v>1571</v>
+      </c>
+      <c r="M99" s="8" t="n">
+        <v>1623</v>
+      </c>
+      <c r="N99" s="8" t="n">
+        <v>1632</v>
+      </c>
+      <c r="O99" s="8" t="n">
+        <v>2228</v>
+      </c>
+      <c r="P99" s="8" t="n">
+        <v>1681</v>
+      </c>
+      <c r="Q99" s="8" t="n">
+        <v>1846</v>
+      </c>
+      <c r="R99" s="8" t="n">
+        <v>2880</v>
+      </c>
+      <c r="S99" s="8" t="n">
+        <v>3570</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Leasehold Improvements</t>
+        </is>
+      </c>
+      <c r="O100" s="8" t="n">
+        <v>2561</v>
+      </c>
+      <c r="P100" s="8" t="n">
+        <v>2375</v>
+      </c>
+      <c r="Q100" s="8" t="n">
+        <v>2439</v>
+      </c>
+      <c r="R100" s="8" t="n">
+        <v>2443</v>
+      </c>
+      <c r="S100" s="8" t="n">
+        <v>2523</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Construction in Progress</t>
         </is>
       </c>
-      <c r="N97" s="8" t="n">
+      <c r="S101" s="8" t="n">
         <v>11187</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>8. INTANGIBLES BY CLASS  ($ in thousands)</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="4" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>8. INTANGIBLES BY CLASS  (mixed: $ in thousands, % / counts as labeled)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
         <is>
           <t>Metric / Segment</t>
         </is>
       </c>
-      <c r="B102" s="5" t="inlineStr">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="C102" s="5" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>Q2 2025</t>
         </is>
       </c>
-      <c r="D102" s="5" t="inlineStr">
+      <c r="D106" s="5" t="inlineStr">
         <is>
           <t>Q3 2025</t>
         </is>
       </c>
-      <c r="E102" s="5" t="inlineStr">
+      <c r="E106" s="5" t="inlineStr">
         <is>
           <t>FY2025</t>
         </is>
       </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="6" t="inlineStr">
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="6" t="inlineStr">
         <is>
           <t>Gross</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="7" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  Customer Relationships</t>
         </is>
       </c>
-      <c r="B104" s="8" t="n">
+      <c r="B108" s="8" t="n">
         <v>13970</v>
       </c>
-      <c r="C104" s="8" t="n">
+      <c r="C108" s="8" t="n">
         <v>126644</v>
       </c>
-      <c r="D104" s="8" t="n">
+      <c r="D108" s="8" t="n">
         <v>132171</v>
       </c>
-      <c r="E104" s="8" t="n">
+      <c r="E108" s="8" t="n">
         <v>132183</v>
       </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="7" t="inlineStr">
+      <c r="F108" s="8" t="n">
+        <v>131865</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  Brands</t>
         </is>
       </c>
-      <c r="B105" s="8" t="n">
+      <c r="B109" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="C105" s="8" t="n">
+      <c r="C109" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="D105" s="8" t="n">
+      <c r="D109" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="E105" s="8" t="n">
+      <c r="E109" s="8" t="n">
         <v>500</v>
       </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="3" t="inlineStr">
+      <c r="F109" s="8" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>X. FILER-SPECIFIC (NOT STANDARDIZED CROSS-TICKER)</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>Hand-curated content from mda_narrative.json. Filer-specific by design.</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="7" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
         <is>
           <t>(empty — populate Ticker Libraries/{TICKER}/MDA and Other/mda_narrative.json)</t>
         </is>

</xml_diff>

<commit_message>
vault backup: 2026-05-10 17:36:04
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_disclosures.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_disclosures.xlsx
@@ -3273,7 +3273,7 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  celh:GeographicalNonNorthAmericaMember</t>
+          <t xml:space="preserve">  Non-North America (rolled up)</t>
         </is>
       </c>
       <c r="V31" s="8" t="n">
@@ -4076,7 +4076,7 @@
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  us-gaap:RestrictedStockMember</t>
+          <t xml:space="preserve">  Restricted Stock</t>
         </is>
       </c>
       <c r="B82" s="8" t="n">
@@ -4086,7 +4086,7 @@
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  celh:StockBasedAwardsIssuedToNonEmployeeConsultantsMember</t>
+          <t xml:space="preserve">  Non-Employee Consultant Awards</t>
         </is>
       </c>
       <c r="D83" s="8" t="n">
@@ -4169,7 +4169,7 @@
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  us-gaap:RestrictedStockMember</t>
+          <t xml:space="preserve">  Restricted Stock</t>
         </is>
       </c>
       <c r="B89" s="8" t="n">

</xml_diff>

<commit_message>
vault backup: 2026-05-16 20:49:31
</commit_message>
<xml_diff>
--- a/Knowledge/Model Outputs/CELH/CELH_disclosures.xlsx
+++ b/Knowledge/Model Outputs/CELH/CELH_disclosures.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rodin\Desktop\Brain\Knowledge\Model Outputs\CELH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AC63B71-B131-4A45-A072-FF7795A951D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F832E7-D5E8-4B09-AEB4-A32DF320700F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="29016" windowHeight="15696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Transcript Reports" sheetId="2" r:id="rId1"/>
@@ -5406,7 +5406,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="160">
   <si>
     <t>CELH -- Structural Disclosure Tables</t>
   </si>
@@ -5811,6 +5811,81 @@
   </si>
   <si>
     <t>Don't think alani is replacing brands but rather category is expanding materially in the subsegment that they serve</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>3Q25</t>
+  </si>
+  <si>
+    <t>Retail Sales Growth</t>
+  </si>
+  <si>
+    <t>Celsisus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combine Market Share of Portfolio </t>
+  </si>
+  <si>
+    <t>YoY</t>
+  </si>
+  <si>
+    <t>Growth</t>
+  </si>
+  <si>
+    <t>Yoy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celsius Brand Scanner Growth </t>
+  </si>
+  <si>
+    <t>Celsius Brand Revenue Growth</t>
+  </si>
+  <si>
+    <t>YTD</t>
+  </si>
+  <si>
+    <t>Celsius Revenue</t>
+  </si>
+  <si>
+    <t>Alani was pretty much the rest</t>
+  </si>
+  <si>
+    <t>Distributor Termination Fee</t>
+  </si>
+  <si>
+    <t>Sales and Marketing (% sales)</t>
+  </si>
+  <si>
+    <t>General and Aministrative (% sales)</t>
+  </si>
+  <si>
+    <t>Yoy growth</t>
+  </si>
+  <si>
+    <t>Quarter Debt reduction</t>
+  </si>
+  <si>
+    <t>Interest Expense reduction</t>
+  </si>
+  <si>
+    <t>4Q25 Forecast</t>
+  </si>
+  <si>
+    <t>23-25%</t>
+  </si>
+  <si>
+    <t>Supply chain not optimized with new Alani integration. Need to optimize co-packing facilities, procurement logistics, greight lanes etc.</t>
+  </si>
+  <si>
+    <t>Basically margin drag on integration of new product lines</t>
+  </si>
+  <si>
+    <t>Expecting margin improvements from Rockstar in 1H26</t>
+  </si>
+  <si>
+    <t>Plan on leaning into international further in 2026</t>
   </si>
 </sst>
 </file>
@@ -5940,7 +6015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -5970,6 +6045,9 @@
     <xf numFmtId="5" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6277,7 +6355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{069CDF8A-BBC4-4C21-BBC9-06CB28FB904C}">
-  <dimension ref="B2:T71"/>
+  <dimension ref="B2:T109"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
@@ -6723,7 +6801,7 @@
         <v>-60.2</v>
       </c>
     </row>
-    <row r="65" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:19" x14ac:dyDescent="0.3">
       <c r="C65" t="s">
         <v>127</v>
       </c>
@@ -6736,7 +6814,7 @@
         <v>189.8</v>
       </c>
     </row>
-    <row r="67" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:19" x14ac:dyDescent="0.3">
       <c r="D67" t="s">
         <v>117</v>
       </c>
@@ -6747,7 +6825,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="68" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:19" x14ac:dyDescent="0.3">
       <c r="C68" t="s">
         <v>130</v>
       </c>
@@ -6761,7 +6839,7 @@
         <v>619.6</v>
       </c>
     </row>
-    <row r="70" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:19" x14ac:dyDescent="0.3">
       <c r="C70" t="s">
         <v>131</v>
       </c>
@@ -6770,12 +6848,239 @@
       </c>
       <c r="E70" s="21"/>
     </row>
-    <row r="71" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:19" x14ac:dyDescent="0.3">
       <c r="C71" t="s">
         <v>133</v>
       </c>
       <c r="D71" s="20">
         <v>1.02</v>
+      </c>
+    </row>
+    <row r="72" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C72" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="75" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B75" t="s">
+        <v>108</v>
+      </c>
+      <c r="C75" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="76" spans="2:19" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="77" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B77" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="C77" s="17">
+        <v>46079</v>
+      </c>
+      <c r="D77" s="16"/>
+      <c r="E77" s="16"/>
+      <c r="F77" s="16"/>
+      <c r="G77" s="16"/>
+      <c r="H77" s="16"/>
+      <c r="I77" s="16"/>
+      <c r="J77" s="16"/>
+      <c r="K77" s="16"/>
+      <c r="L77" s="16"/>
+      <c r="M77" s="16"/>
+      <c r="N77" s="16"/>
+      <c r="O77" s="16"/>
+      <c r="P77" s="16"/>
+      <c r="Q77" s="16"/>
+      <c r="R77" s="16"/>
+      <c r="S77" s="16"/>
+    </row>
+    <row r="78" spans="2:19" ht="3" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C78" s="13"/>
+      <c r="D78" s="15"/>
+      <c r="E78" s="15"/>
+      <c r="F78" s="15"/>
+      <c r="G78" s="15"/>
+      <c r="H78" s="15"/>
+      <c r="I78" s="15"/>
+      <c r="J78" s="15"/>
+      <c r="K78" s="15"/>
+      <c r="L78" s="15"/>
+      <c r="M78" s="15"/>
+      <c r="N78" s="15"/>
+      <c r="O78" s="15"/>
+      <c r="P78" s="15"/>
+      <c r="Q78" s="15"/>
+      <c r="R78" s="15"/>
+      <c r="S78" s="15"/>
+    </row>
+    <row r="80" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C80" t="s">
+        <v>137</v>
+      </c>
+      <c r="D80" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="81" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C81" t="s">
+        <v>138</v>
+      </c>
+      <c r="D81" s="20">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="82" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C82" t="s">
+        <v>115</v>
+      </c>
+      <c r="D82" s="20">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="E82" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="84" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="D84" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="85" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C85" t="s">
+        <v>139</v>
+      </c>
+      <c r="D85" s="20">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="86" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C86" t="s">
+        <v>141</v>
+      </c>
+      <c r="D86" s="20">
+        <v>0.31</v>
+      </c>
+      <c r="E86" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="89" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C89" t="s">
+        <v>143</v>
+      </c>
+      <c r="D89" s="20">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="90" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C90" t="s">
+        <v>144</v>
+      </c>
+      <c r="D90" s="20">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="92" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="D92" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="93" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C93" t="s">
+        <v>146</v>
+      </c>
+      <c r="D93" s="20">
+        <v>0.12</v>
+      </c>
+      <c r="E93" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="95" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="D95" t="s">
+        <v>136</v>
+      </c>
+      <c r="E95" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="96" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C96" t="s">
+        <v>148</v>
+      </c>
+      <c r="D96" s="19">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="97" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C97" t="s">
+        <v>149</v>
+      </c>
+      <c r="D97" s="20">
+        <v>0.2</v>
+      </c>
+      <c r="E97" s="27" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="98" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="D98" s="20"/>
+    </row>
+    <row r="99" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C99" t="s">
+        <v>150</v>
+      </c>
+      <c r="D99" s="20">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="100" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C100" t="s">
+        <v>151</v>
+      </c>
+      <c r="D100" s="20">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="102" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C102" t="s">
+        <v>152</v>
+      </c>
+      <c r="D102" s="19">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="103" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C103" t="s">
+        <v>153</v>
+      </c>
+      <c r="D103" s="19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="105" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C105" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="106" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C106" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="107" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C107" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="108" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C108" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="109" spans="3:5" x14ac:dyDescent="0.3">
+      <c r="C109" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>